<commit_message>
Add Monthly Breakdown tab; first-names-only across workbook
- New 'Monthly Breakdown' tab: Apr-Aug month x defect matrix per tissue x
  slaughterhouse x part combo (Martins 541/506, Parks 518 and 541 separate,
  Nahunta pelvic 541, Nahunta thoracic 521). Two overview matrices (FPY and
  fails by month) + a detail block per combo: live SUMPRODUCT volume rows off
  the Inspection Log, FPY heatmaps, and issues normalized into 9 standard
  defect categories (urethra/bladder, membrane, bowel, short/mesentery,
  critical-area, ureter, lung, heart, other). All 166 fails categorized and
  verified (167 tags incl. the known 8/12 thoracic breakdown +1; caveats noted
  on-sheet).
- Scrub last names workbook-wide (log, notes, SmartAssessment strings): first
  names only. Deck already clean.
- README: new tab documented, first-name convention, category-tagging step.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/SH_IQC_Inspections.xlsx
+++ b/QC inspections suppliers/SH_IQC_Inspections.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Slaughterhouse IQC" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Quality Dashboard" sheetId="14" state="visible" r:id="rId17"/>
+    <sheet name="Monthly Breakdown" sheetId="15" state="visible" r:id="rId18"/>
     <sheet name="SmartAssessment" sheetId="12" state="visible" r:id="rId15"/>
     <sheet name="Defect Atlas" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="README" sheetId="10" state="visible" r:id="rId12"/>
@@ -188,7 +189,7 @@
     <t xml:space="preserve">Martins</t>
   </si>
   <si>
-    <t xml:space="preserve">Toni Cruz</t>
+    <t xml:space="preserve">Toni</t>
   </si>
   <si>
     <t xml:space="preserve">Jesus</t>
@@ -260,7 +261,7 @@
     <t xml:space="preserve">Parks Family Meats</t>
   </si>
   <si>
-    <t xml:space="preserve">Rasmin Mujanovic</t>
+    <t xml:space="preserve">Rasmin</t>
   </si>
   <si>
     <t xml:space="preserve">Natalie</t>
@@ -335,7 +336,7 @@
     <t xml:space="preserve">1 hole in bowel; 1 label marked for thin area in bowel</t>
   </si>
   <si>
-    <t xml:space="preserve">Toni Cruz / Jesus</t>
+    <t xml:space="preserve">Toni / Jesus</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-15</t>
@@ -407,7 +408,7 @@
     <t xml:space="preserve">4 mesentery length too short in critical zone; 1 bladder damage (internals exposed)</t>
   </si>
   <si>
-    <t xml:space="preserve">Rasmin Mujanovic / Natalie</t>
+    <t xml:space="preserve">Rasmin / Natalie</t>
   </si>
   <si>
     <t xml:space="preserve">2026-06-01</t>
@@ -539,7 +540,7 @@
     <t xml:space="preserve">10. New slaughterhouse &amp; inspection team (Parks, 05/28)</t>
   </si>
   <si>
-    <t xml:space="preserve">First SH-floor inspection at Parks Family Meats, with a new ATM inspector (Rasmin Mujanovic) and new SH tech (Natalie) vs. Toni Cruz / Jesus at Martins. Source PN was written 668518 and normalized to 666518 (per the workbook's typo convention). No batch/lot was recorded ('no batch data'), so this visit has no SH→ATM link, and the related Parks ATM lot 5502428883 (7 received / 7 scrapped, 'before our visit') has no SH-floor counterpart here. Date taken from the source date field (05/28); the carried-over note text mentioning '5/27' and non-intact labels does not apply to this intact-only Parks visit.</t>
+    <t xml:space="preserve">First SH-floor inspection at Parks Family Meats, with a new ATM inspector (Rasmin) and new SH tech (Natalie) vs. Toni / Jesus at Martins. Source PN was written 668518 and normalized to 666518 (per the workbook's typo convention). No batch/lot was recorded ('no batch data'), so this visit has no SH→ATM link, and the related Parks ATM lot 5502428883 (7 received / 7 scrapped, 'before our visit') has no SH-floor counterpart here. Date taken from the source date field (05/28); the carried-over note text mentioning '5/27' and non-intact labels does not apply to this intact-only Parks visit.</t>
   </si>
   <si>
     <t xml:space="preserve">11. Visit 7 harvest-date split (06/01 vs 06/03)</t>
@@ -3020,6 +3021,1868 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G99"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="true">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monthly Breakdown — Inspections by Tissue × Slaughterhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="58" customHeight="true">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Month-by-month view of every tissue-type / slaughterhouse / part combination: volumes, first-pass yield, and the issues found (scrap reasons normalized into standard defect categories). Apr–Aug 2026. Volume rows are live formulas over the Inspection Log; defect counts are analyst-categorized from the scrap notes (see notes at bottom).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="18" customHeight="true">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OVERVIEW — FIRST-PASS YIELD BY MONTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tissue @ SH · Part</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">July</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Martins · 666541</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C6" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D6" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E6" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F6" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G6" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Martins · 666506</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C7" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D7" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E7" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F7" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G7" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Parks · 666518</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C8" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D8" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E8" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F8" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G8" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Parks · 666541</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C9" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D9" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E9" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F9" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G9" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Nahunta · 666541</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C10" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D10" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E10" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F10" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G10" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thoracic @ Nahunta · 666521</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C11" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D11" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E11" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F11" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G11" s="15" t="n">
+        <f aca="false">IF(SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64)/SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13" ht="18" customHeight="true">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OVERVIEW — ISSUES FOUND (# FAILED) BY MONTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tissue @ SH · Part</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">July</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Martins · 666541</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C15" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D15" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E15" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F15" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G15" s="6" t="n">
+        <f aca="false">SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64)</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Martins · 666506</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C16" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D16" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E16" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F16" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G16" s="6" t="n">
+        <f aca="false">SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64)</f>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Parks · 666518</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C17" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D17" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E17" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F17" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G17" s="6" t="n">
+        <f aca="false">SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64)</f>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Parks · 666541</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C18" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D18" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E18" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F18" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G18" s="6" t="n">
+        <f aca="false">SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64)</f>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic @ Nahunta · 666541</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C19" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D19" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E19" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F19" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G19" s="6" t="n">
+        <f aca="false">SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64)</f>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thoracic @ Nahunta · 666521</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C20" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D20" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E20" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F20" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G20" s="6" t="n">
+        <f aca="false">SUMPRODUCT(('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64)</f>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="18" customHeight="true">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PELVIC @ MARTINS — 666541 (intact)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metric</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">July</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Inspected</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C24" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D24" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E24" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F24" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G24" s="6" t="n">
+        <f aca="false">SUM(B24:F24)</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Pass</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="C25" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="D25" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="E25" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="F25" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="G25" s="6" t="n">
+        <f aca="false">SUM(B25:F25)</f>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Fail</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C26" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D26" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E26" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F26" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G26" s="6" t="n">
+        <f aca="false">SUM(B26:F26)</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-Pass Yield</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <f aca="false">IF(B24="","",IF(B24=0,"",B25/B24))</f>
+      </c>
+      <c r="C27" s="15" t="n">
+        <f aca="false">IF(C24="","",IF(C24=0,"",C25/C24))</f>
+      </c>
+      <c r="D27" s="15" t="n">
+        <f aca="false">IF(D24="","",IF(D24=0,"",D25/D24))</f>
+      </c>
+      <c r="E27" s="15" t="n">
+        <f aca="false">IF(E24="","",IF(E24=0,"",E25/E24))</f>
+      </c>
+      <c r="F27" s="15" t="n">
+        <f aca="false">IF(F24="","",IF(F24=0,"",F25/F24))</f>
+      </c>
+      <c r="G27" s="15" t="n">
+        <f aca="false">IF(G24=0,"",G25/G24)</f>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="true">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Issues found (defect category counts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Urethra / bladder damage</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Membrane damage</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Bowel damage / separation</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Short block / mesentery length</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Other / unspecified</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total issues</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <f aca="false">IF(SUM(B29:B33)=0,"",SUM(B29:B33))</f>
+      </c>
+      <c r="C34" s="6" t="n">
+        <f aca="false">IF(SUM(C29:C33)=0,"",SUM(C29:C33))</f>
+      </c>
+      <c r="D34" s="6" t="n">
+        <f aca="false">IF(SUM(D29:D33)=0,"",SUM(D29:D33))</f>
+      </c>
+      <c r="E34" s="6" t="n">
+        <f aca="false">IF(SUM(E29:E33)=0,"",SUM(E29:E33))</f>
+      </c>
+      <c r="F34" s="6" t="n">
+        <f aca="false">IF(SUM(F29:F33)=0,"",SUM(F29:F33))</f>
+      </c>
+      <c r="G34" s="6" t="n">
+        <f aca="false">SUM(G29:G33)</f>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36" ht="18" customHeight="true">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PELVIC @ MARTINS — 666506 (non-intact)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metric</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">July</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Inspected</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C38" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D38" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E38" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F38" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G38" s="6" t="n">
+        <f aca="false">SUM(B38:F38)</f>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Pass</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="C39" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="D39" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="E39" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="F39" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="G39" s="6" t="n">
+        <f aca="false">SUM(B39:F39)</f>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Fail</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C40" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D40" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E40" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F40" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Martins")*('Slaughterhouse IQC'!$F$6:$F$64="666506")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G40" s="6" t="n">
+        <f aca="false">SUM(B40:F40)</f>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-Pass Yield</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="n">
+        <f aca="false">IF(B38="","",IF(B38=0,"",B39/B38))</f>
+      </c>
+      <c r="C41" s="15" t="n">
+        <f aca="false">IF(C38="","",IF(C38=0,"",C39/C38))</f>
+      </c>
+      <c r="D41" s="15" t="n">
+        <f aca="false">IF(D38="","",IF(D38=0,"",D39/D38))</f>
+      </c>
+      <c r="E41" s="15" t="n">
+        <f aca="false">IF(E38="","",IF(E38=0,"",E39/E38))</f>
+      </c>
+      <c r="F41" s="15" t="n">
+        <f aca="false">IF(F38="","",IF(F38=0,"",F39/F38))</f>
+      </c>
+      <c r="G41" s="15" t="n">
+        <f aca="false">IF(G38=0,"",G39/G38)</f>
+      </c>
+    </row>
+    <row r="42" ht="15" customHeight="true">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Issues found (defect category counts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Urethra / bladder damage</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G43" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Membrane damage</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Bowel damage / separation</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Short block / mesentery length</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Other / unspecified</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total issues</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="n">
+        <f aca="false">IF(SUM(B43:B47)=0,"",SUM(B43:B47))</f>
+      </c>
+      <c r="C48" s="6" t="n">
+        <f aca="false">IF(SUM(C43:C47)=0,"",SUM(C43:C47))</f>
+      </c>
+      <c r="D48" s="6" t="n">
+        <f aca="false">IF(SUM(D43:D47)=0,"",SUM(D43:D47))</f>
+      </c>
+      <c r="E48" s="6" t="n">
+        <f aca="false">IF(SUM(E43:E47)=0,"",SUM(E43:E47))</f>
+      </c>
+      <c r="F48" s="6" t="n">
+        <f aca="false">IF(SUM(F43:F47)=0,"",SUM(F43:F47))</f>
+      </c>
+      <c r="G48" s="6" t="n">
+        <f aca="false">SUM(G43:G47)</f>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50" ht="18" customHeight="true">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PELVIC @ PARKS — 666518 (intact, SM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metric</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">July</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Inspected</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C52" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D52" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E52" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F52" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G52" s="6" t="n">
+        <f aca="false">SUM(B52:F52)</f>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Pass</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="C53" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="D53" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="E53" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="F53" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="G53" s="6" t="n">
+        <f aca="false">SUM(B53:F53)</f>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Fail</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C54" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D54" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E54" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F54" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666518")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G54" s="6" t="n">
+        <f aca="false">SUM(B54:F54)</f>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-Pass Yield</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="n">
+        <f aca="false">IF(B52="","",IF(B52=0,"",B53/B52))</f>
+      </c>
+      <c r="C55" s="15" t="n">
+        <f aca="false">IF(C52="","",IF(C52=0,"",C53/C52))</f>
+      </c>
+      <c r="D55" s="15" t="n">
+        <f aca="false">IF(D52="","",IF(D52=0,"",D53/D52))</f>
+      </c>
+      <c r="E55" s="15" t="n">
+        <f aca="false">IF(E52="","",IF(E52=0,"",E53/E52))</f>
+      </c>
+      <c r="F55" s="15" t="n">
+        <f aca="false">IF(F52="","",IF(F52=0,"",F53/F52))</f>
+      </c>
+      <c r="G55" s="15" t="n">
+        <f aca="false">IF(G52=0,"",G53/G52)</f>
+      </c>
+    </row>
+    <row r="56" ht="15" customHeight="true">
+      <c r="A56" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Issues found (defect category counts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Urethra / bladder damage</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G57" s="6" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Bowel damage / separation</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Short block / mesentery length</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Critical-area laceration</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G60" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Ureter damage</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total issues</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="n">
+        <f aca="false">IF(SUM(B57:B61)=0,"",SUM(B57:B61))</f>
+      </c>
+      <c r="C62" s="6" t="n">
+        <f aca="false">IF(SUM(C57:C61)=0,"",SUM(C57:C61))</f>
+      </c>
+      <c r="D62" s="6" t="n">
+        <f aca="false">IF(SUM(D57:D61)=0,"",SUM(D57:D61))</f>
+      </c>
+      <c r="E62" s="6" t="n">
+        <f aca="false">IF(SUM(E57:E61)=0,"",SUM(E57:E61))</f>
+      </c>
+      <c r="F62" s="6" t="n">
+        <f aca="false">IF(SUM(F57:F61)=0,"",SUM(F57:F61))</f>
+      </c>
+      <c r="G62" s="6" t="n">
+        <f aca="false">SUM(G57:G61)</f>
+      </c>
+    </row>
+    <row r="63"/>
+    <row r="64" ht="18" customHeight="true">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PELVIC @ PARKS — 666541 (intact — spec transition, from 08/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metric</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">July</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August</t>
+        </is>
+      </c>
+      <c r="G65" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Inspected</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C66" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D66" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E66" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F66" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G66" s="6" t="n">
+        <f aca="false">SUM(B66:F66)</f>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Pass</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="C67" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="D67" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="E67" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="F67" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="G67" s="6" t="n">
+        <f aca="false">SUM(B67:F67)</f>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Fail</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C68" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D68" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E68" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F68" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Parks Family Meats")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G68" s="6" t="n">
+        <f aca="false">SUM(B68:F68)</f>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-Pass Yield</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="n">
+        <f aca="false">IF(B66="","",IF(B66=0,"",B67/B66))</f>
+      </c>
+      <c r="C69" s="15" t="n">
+        <f aca="false">IF(C66="","",IF(C66=0,"",C67/C66))</f>
+      </c>
+      <c r="D69" s="15" t="n">
+        <f aca="false">IF(D66="","",IF(D66=0,"",D67/D66))</f>
+      </c>
+      <c r="E69" s="15" t="n">
+        <f aca="false">IF(E66="","",IF(E66=0,"",E67/E66))</f>
+      </c>
+      <c r="F69" s="15" t="n">
+        <f aca="false">IF(F66="","",IF(F66=0,"",F67/F66))</f>
+      </c>
+      <c r="G69" s="15" t="n">
+        <f aca="false">IF(G66=0,"",G67/G66)</f>
+      </c>
+    </row>
+    <row r="70" ht="15" customHeight="true">
+      <c r="A70" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Issues found (defect category counts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Bowel damage / separation</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total issues</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="n">
+        <f aca="false">IF(SUM(B71:B71)=0,"",SUM(B71:B71))</f>
+      </c>
+      <c r="C72" s="6" t="n">
+        <f aca="false">IF(SUM(C71:C71)=0,"",SUM(C71:C71))</f>
+      </c>
+      <c r="D72" s="6" t="n">
+        <f aca="false">IF(SUM(D71:D71)=0,"",SUM(D71:D71))</f>
+      </c>
+      <c r="E72" s="6" t="n">
+        <f aca="false">IF(SUM(E71:E71)=0,"",SUM(E71:E71))</f>
+      </c>
+      <c r="F72" s="6" t="n">
+        <f aca="false">IF(SUM(F71:F71)=0,"",SUM(F71:F71))</f>
+      </c>
+      <c r="G72" s="6" t="n">
+        <f aca="false">SUM(G71:G71)</f>
+      </c>
+    </row>
+    <row r="73"/>
+    <row r="74" ht="18" customHeight="true">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PELVIC @ NAHUNTA — 666541 (intact — side line)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metric</t>
+        </is>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
+      <c r="D75" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">July</t>
+        </is>
+      </c>
+      <c r="F75" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August</t>
+        </is>
+      </c>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Inspected</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C76" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D76" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E76" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F76" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G76" s="6" t="n">
+        <f aca="false">SUM(B76:F76)</f>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Pass</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="C77" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="D77" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="E77" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="F77" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="G77" s="6" t="n">
+        <f aca="false">SUM(B77:F77)</f>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Fail</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C78" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D78" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E78" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F78" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666541")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G78" s="6" t="n">
+        <f aca="false">SUM(B78:F78)</f>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-Pass Yield</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="n">
+        <f aca="false">IF(B76="","",IF(B76=0,"",B77/B76))</f>
+      </c>
+      <c r="C79" s="15" t="n">
+        <f aca="false">IF(C76="","",IF(C76=0,"",C77/C76))</f>
+      </c>
+      <c r="D79" s="15" t="n">
+        <f aca="false">IF(D76="","",IF(D76=0,"",D77/D76))</f>
+      </c>
+      <c r="E79" s="15" t="n">
+        <f aca="false">IF(E76="","",IF(E76=0,"",E77/E76))</f>
+      </c>
+      <c r="F79" s="15" t="n">
+        <f aca="false">IF(F76="","",IF(F76=0,"",F77/F76))</f>
+      </c>
+      <c r="G79" s="15" t="n">
+        <f aca="false">IF(G76=0,"",G77/G76)</f>
+      </c>
+    </row>
+    <row r="80" ht="15" customHeight="true">
+      <c r="A80" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Issues found (defect category counts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Other / unspecified</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G81" s="6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total issues</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="n">
+        <f aca="false">IF(SUM(B81:B81)=0,"",SUM(B81:B81))</f>
+      </c>
+      <c r="C82" s="6" t="n">
+        <f aca="false">IF(SUM(C81:C81)=0,"",SUM(C81:C81))</f>
+      </c>
+      <c r="D82" s="6" t="n">
+        <f aca="false">IF(SUM(D81:D81)=0,"",SUM(D81:D81))</f>
+      </c>
+      <c r="E82" s="6" t="n">
+        <f aca="false">IF(SUM(E81:E81)=0,"",SUM(E81:E81))</f>
+      </c>
+      <c r="F82" s="6" t="n">
+        <f aca="false">IF(SUM(F81:F81)=0,"",SUM(F81:F81))</f>
+      </c>
+      <c r="G82" s="6" t="n">
+        <f aca="false">SUM(G81:G81)</f>
+      </c>
+    </row>
+    <row r="83"/>
+    <row r="84" ht="18" customHeight="true">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">THORACIC @ NAHUNTA — 666521 (lung / heart)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metric</t>
+        </is>
+      </c>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">April</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June</t>
+        </is>
+      </c>
+      <c r="E85" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">July</t>
+        </is>
+      </c>
+      <c r="F85" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August</t>
+        </is>
+      </c>
+      <c r="G85" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Inspected</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="C86" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="D86" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="E86" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="F86" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64))</f>
+      </c>
+      <c r="G86" s="6" t="n">
+        <f aca="false">SUM(B86:F86)</f>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Pass</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="C87" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="D87" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="E87" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="F87" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$J$6:$J$64))</f>
+      </c>
+      <c r="G87" s="6" t="n">
+        <f aca="false">SUM(B87:F87)</f>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Fail</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-04")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="C88" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-05")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="D88" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-06")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="E88" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-07")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="F88" s="6" t="n">
+        <f aca="false">IF(SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$I$6:$I$64)=0,"",SUMPRODUCT((LEFT('Slaughterhouse IQC'!$A$6:$A$64,7)="2026-08")*('Slaughterhouse IQC'!$B$6:$B$64="Nahunta")*('Slaughterhouse IQC'!$F$6:$F$64="666521")*'Slaughterhouse IQC'!$K$6:$K$64))</f>
+      </c>
+      <c r="G88" s="6" t="n">
+        <f aca="false">SUM(B88:F88)</f>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-Pass Yield</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="n">
+        <f aca="false">IF(B86="","",IF(B86=0,"",B87/B86))</f>
+      </c>
+      <c r="C89" s="15" t="n">
+        <f aca="false">IF(C86="","",IF(C86=0,"",C87/C86))</f>
+      </c>
+      <c r="D89" s="15" t="n">
+        <f aca="false">IF(D86="","",IF(D86=0,"",D87/D86))</f>
+      </c>
+      <c r="E89" s="15" t="n">
+        <f aca="false">IF(E86="","",IF(E86=0,"",E87/E86))</f>
+      </c>
+      <c r="F89" s="15" t="n">
+        <f aca="false">IF(F86="","",IF(F86=0,"",F87/F86))</f>
+      </c>
+      <c r="G89" s="15" t="n">
+        <f aca="false">IF(G86=0,"",G87/G86)</f>
+      </c>
+    </row>
+    <row r="90" ht="15" customHeight="true">
+      <c r="A90" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Issues found (defect category counts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Lung laceration</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="G91" s="6" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Heart damage</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="G92" s="6" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total issues</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="n">
+        <f aca="false">IF(SUM(B91:B92)=0,"",SUM(B91:B92))</f>
+      </c>
+      <c r="C93" s="6" t="n">
+        <f aca="false">IF(SUM(C91:C92)=0,"",SUM(C91:C92))</f>
+      </c>
+      <c r="D93" s="6" t="n">
+        <f aca="false">IF(SUM(D91:D92)=0,"",SUM(D91:D92))</f>
+      </c>
+      <c r="E93" s="6" t="n">
+        <f aca="false">IF(SUM(E91:E92)=0,"",SUM(E91:E92))</f>
+      </c>
+      <c r="F93" s="6" t="n">
+        <f aca="false">IF(SUM(F91:F92)=0,"",SUM(F91:F92))</f>
+      </c>
+      <c r="G93" s="6" t="n">
+        <f aca="false">SUM(G91:G92)</f>
+      </c>
+    </row>
+    <row r="94"/>
+    <row r="95" ht="18" customHeight="true">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="44" customHeight="true">
+      <c r="A96" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Defect categories normalize free-text scrap reasons: blood clots and 'damaged after cleaning' → Other; bowel-cleaning bursts and bowel/colon–mesentery separations → Bowel damage / separation; mesentery holes/lacerations in the critical area → Critical-area laceration; 'small bladder' / 'deformed bladder' → Urethra / bladder. Original wording stays in the Inspection Log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="44" customHeight="true">
+      <c r="A97" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Volume rows (# Inspected / Pass / Fail, FPY) are live formulas over the Inspection Log (rows 6–64) — they update automatically when the log grows within that range. Defect-category counts are analyst-tagged from scrap notes (static snapshot through 08/19); retag new rows when appending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="44" customHeight="true">
+      <c r="A98" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Known count caveats: Nahunta thoracic 8/12 defect breakdown sums to 12 vs 11 recorded fails (kept as written, so thoracic categorized issues = 50 vs 49 fails in August). Nahunta pelvic 8/12 (13/1/12) has no defect breakdown and is provisional → all 12 in Other/unspecified. Martins 666541 7/20 includes 1 undocumented reject (Other).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="44" customHeight="true">
+      <c r="A99" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Parks runs as two part lines across the spec transition: 666518 through 07/30, 666541 from 08/10 — shown separately by request. Nahunta pelvic is a side line (thoracic is the primary part there).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A56:G56"/>
+    <mergeCell ref="A64:G64"/>
+    <mergeCell ref="A70:G70"/>
+    <mergeCell ref="A74:G74"/>
+    <mergeCell ref="A80:G80"/>
+    <mergeCell ref="A84:G84"/>
+    <mergeCell ref="A90:G90"/>
+    <mergeCell ref="A95:G95"/>
+    <mergeCell ref="A96:G96"/>
+    <mergeCell ref="A97:G97"/>
+    <mergeCell ref="A98:G98"/>
+    <mergeCell ref="A99:G99"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6:G11 B27:G27 B41:G41 B55:G55 B69:G69 B79:G79 B89:G89">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0.3"/>
+        <cfvo type="num" val="0.8"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M100"/>
@@ -3140,7 +5003,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -3199,7 +5062,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -3258,7 +5121,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -3317,7 +5180,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -3376,7 +5239,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -3435,7 +5298,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -3494,7 +5357,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -3553,7 +5416,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -3612,7 +5475,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -3671,7 +5534,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -3730,7 +5593,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -3789,7 +5652,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -3848,7 +5711,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -3907,7 +5770,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -3966,7 +5829,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -4025,7 +5888,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -4084,7 +5947,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -4143,7 +6006,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -4202,7 +6065,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -4261,7 +6124,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -4320,7 +6183,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -4379,7 +6242,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -4438,7 +6301,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -4497,7 +6360,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -4556,7 +6419,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -4615,7 +6478,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -4674,7 +6537,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -4733,7 +6596,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -4792,7 +6655,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -4851,7 +6714,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -4910,7 +6773,7 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -4969,7 +6832,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -5028,7 +6891,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -5087,7 +6950,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -5146,7 +7009,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -5205,7 +7068,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
@@ -5264,7 +7127,7 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
@@ -5323,7 +7186,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -5382,7 +7245,7 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -5441,7 +7304,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -5500,7 +7363,7 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -5559,7 +7422,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -5618,7 +7481,7 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -5677,7 +7540,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -5741,7 +7604,7 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jordan Guthrie</t>
+          <t xml:space="preserve">Jordan</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -5800,7 +7663,7 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jordan Guthrie</t>
+          <t xml:space="preserve">Jordan</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -5854,7 +7717,7 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -5913,7 +7776,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -5977,7 +7840,7 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jordan Guthrie</t>
+          <t xml:space="preserve">Jordan</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -6031,7 +7894,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -6090,7 +7953,7 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -6149,7 +8012,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -6208,7 +8071,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -6272,7 +8135,7 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jordan Guthrie</t>
+          <t xml:space="preserve">Jordan</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -6331,7 +8194,7 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jordan Guthrie</t>
+          <t xml:space="preserve">Jordan</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -6385,7 +8248,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic</t>
+          <t xml:space="preserve">Rasmin</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -6444,7 +8307,7 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -6503,7 +8366,7 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toni Cruz</t>
+          <t xml:space="preserve">Toni</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
@@ -6567,7 +8430,7 @@
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jordan Guthrie</t>
+          <t xml:space="preserve">Jordan</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -6839,7 +8702,7 @@
       </c>
       <c r="B85" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">First SH-floor inspection at Parks Family Meats, with a new ATM inspector (Rasmin Mujanovic) and new SH tech (Natalie) vs. Toni Cruz / Jesus at Martins. Source PN was written 668518 and normalized to 666518 (per the workbook's typo convention). No batch/lot was recorded ('no batch data'), so this visit has no SH→ATM link, and the related Parks ATM lot 5502428883 (7 received / 7 scrapped, 'before our visit') has no SH-floor counterpart here. Date taken from the source date field (05/28); the carried-over note text mentioning '5/27' and non-intact labels does not apply to this intact-only Parks visit.</t>
+          <t xml:space="preserve">First SH-floor inspection at Parks Family Meats, with a new ATM inspector (Rasmin) and new SH tech (Natalie) vs. Toni / Jesus at Martins. Source PN was written 668518 and normalized to 666518 (per the workbook's typo convention). No batch/lot was recorded ('no batch data'), so this visit has no SH→ATM link, and the related Parks ATM lot 5502428883 (7 received / 7 scrapped, 'before our visit') has no SH-floor counterpart here. Date taken from the source date field (05/28); the carried-over note text mentioning '5/27' and non-intact labels does not apply to this intact-only Parks visit.</t>
         </is>
       </c>
     </row>
@@ -6935,7 +8798,7 @@
       </c>
       <c r="B93" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visit 15 = 06/29 Martins; Visit 16 = 06/29 Parks; Visit 17 = 07/06 Martins; Visit 18 = 07/13 Martins; Visit 19 = 07/13 Parks. DATA-ACCURACY FIX: on both Parks sheets the source “# Fail” cell undercounted because blocks damaged during bowel-cleaning were written in the notes but not added to the fail tally. Corrected to inspected − pass, which matches the scrap breakdown — Visit 16 (06/29) = 50/38/12 (source cell read 10; 2 cleaning-damage + 2 short + 1 critical + 7 urethra/bladder = 12); Visit 19 (07/13) = 34/29/5 (source cell read 3; 2 cleaning-damage + 3 short = 5). Visit 17 (07/06) reuses Visit 15’s lots 5502471460/5502471457 — a tally-sheet carry-over recorded as a separate visit (see note 9). Visit 18’s inspector field was blank on the source; recorded as Toni Cruz, the standing Martins inspector.</t>
+          <t xml:space="preserve">Visit 15 = 06/29 Martins; Visit 16 = 06/29 Parks; Visit 17 = 07/06 Martins; Visit 18 = 07/13 Martins; Visit 19 = 07/13 Parks. DATA-ACCURACY FIX: on both Parks sheets the source “# Fail” cell undercounted because blocks damaged during bowel-cleaning were written in the notes but not added to the fail tally. Corrected to inspected − pass, which matches the scrap breakdown — Visit 16 (06/29) = 50/38/12 (source cell read 10; 2 cleaning-damage + 2 short + 1 critical + 7 urethra/bladder = 12); Visit 19 (07/13) = 34/29/5 (source cell read 3; 2 cleaning-damage + 3 short = 5). Visit 17 (07/06) reuses Visit 15’s lots 5502471460/5502471457 — a tally-sheet carry-over recorded as a separate visit (see note 9). Visit 18’s inspector field was blank on the source; recorded as Toni, the standing Martins inspector.</t>
         </is>
       </c>
     </row>
@@ -6959,7 +8822,7 @@
       </c>
       <c r="B95" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visit 20 = 07/20 Martins (reuses Visit 18 lots 5502495107 / 5502495104 — carry-over); Visit 21 = 07/27 Martins (new lots 5502512228 / 5502512225); Visit 22 = 07/29 Nahunta — the first THORACIC (PN 666521, lot 5502512218), a new product family at a new slaughterhouse with a new inspector/tech (Kris / Jordan Guthrie), 19 inspected / 6 pass / 13 fail (31.6%); Visit 23 = 07/30 Parks (666518, majority-male pigs noted). The thoracic is logged in the raw data and summarized on the "Quality Summary by Part" tab, but is EXCLUDED from the pelvic-block rollup, TOTAL and SH→ATM sections so pelvic yield stays comparable across a single product family.</t>
+          <t xml:space="preserve">Visit 20 = 07/20 Martins (reuses Visit 18 lots 5502495107 / 5502495104 — carry-over); Visit 21 = 07/27 Martins (new lots 5502512228 / 5502512225); Visit 22 = 07/29 Nahunta — the first THORACIC (PN 666521, lot 5502512218), a new product family at a new slaughterhouse with a new inspector/tech (Kris / Jordan), 19 inspected / 6 pass / 13 fail (31.6%); Visit 23 = 07/30 Parks (666518, majority-male pigs noted). The thoracic is logged in the raw data and summarized on the "Quality Summary by Part" tab, but is EXCLUDED from the pelvic-block rollup, TOTAL and SH→ATM sections so pelvic yield stays comparable across a single product family.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 'SH vs ATM Issues' tab: historical defect profiles per tissue
Side-by-side per tissue (Pelvic, Thoracic): SH defect categories from the
Inspection Log vs ATM SAP reason-code totals (net 551/552), with 2026 and
all-time columns, data bars, and quality-only subtotals excluding planned
withdrawals (1220 Destructive Testing, 9991 R&D, 9994 Line Clearance - marked *).

Code labels decoded per Quality: 1220 = Destructive Testing (eng/R&D use),
7 = Others, 1201 = Tech Performance; legacy 4/5/1 remain unmapped. Updated the
1220 label + caveat on the SH vs ATM by Batch tab accordingly.

Alignment reads: pelvic ATM scrap is 52% Laceration/Cut mirroring SH cut
damage (55 of 104 SH fails); blood clots/received damage are ATM-only finds.
Thoracic 2026 quality scrap ~50% of received (434/869) - both stages say
lacerations, confirming harvesting-side origin.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/SH_IQC_Inspections.xlsx
+++ b/QC inspections suppliers/SH_IQC_Inspections.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Quality Dashboard" sheetId="14" r:id="rId2"/>
     <sheet name="Monthly Breakdown" sheetId="15" r:id="rId3"/>
     <sheet name="SH vs ATM by Batch" sheetId="21" r:id="rId16"/>
+    <sheet name="SH vs ATM Issues" sheetId="22" r:id="rId17"/>
     <sheet name="Apr 2026" sheetId="16" r:id="rId4"/>
     <sheet name="May 2026" sheetId="17" r:id="rId5"/>
     <sheet name="Jun 2026" sheetId="18" r:id="rId6"/>
@@ -7361,7 +7362,7 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1220 (unmapped — confirm label)</t>
+          <t xml:space="preserve">1220 Destructive Testing (eng/R&amp;D)</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
@@ -7564,7 +7565,7 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">(unmapped — confirm label) ●</t>
+          <t xml:space="preserve">Destructive Testing (eng/R&amp;D) ●</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -7929,7 +7930,7 @@
     <row r="56" ht="44" customHeight="1">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Caveats: code 1220 (5 units, lot 5502471460) is not in the provided legend — confirm its label. 9991 R&amp;D/Testing (10 units, lot 5502404928) is a planned withdrawal, not a quality defect. Lot 5502523283 also carried a small Nahunta pelvic line at SH; the ATM batch is thoracic material only. Lot 5502523269 (received 8/05) has no scrap postings yet.</t>
+          <t xml:space="preserve">• Caveats: code 1220 = Destructive Testing (engineering/R&amp;D use) — a planned withdrawal, not a quality defect (5 units, lot 5502471460); same for 9991 R&amp;D/Testing (10 units, lot 5502404928). Lot 5502523283 also carried a small Nahunta pelvic line at SH; the ATM batch is thoracic material only. Lot 5502523269 (received 8/05) has no scrap postings yet.</t>
         </is>
       </c>
     </row>
@@ -8008,6 +8009,785 @@
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF638EC6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L43"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="3" width="11" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="3" customWidth="1"/>
+    <col min="7" max="9" width="11" customWidth="1"/>
+    <col min="10" max="12" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH Issues vs ATM Issues — by Tissue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What fails at the slaughterhouse floor vs what gets scrapped at ATM, per tissue. SH side: analyst-categorized scrap reasons from the Inspection Log (Apr–Aug 2026; pelvic = all parts 666541/666506/666518, thoracic = 666521). ATM side: SAP reason-code totals net of reversals (551/552) for the materials ATM tracks (pelvic 666541, thoracic 666521) — shown for 2026 and all-time (thoracic history reaches back to Jul 2024). * = planned/process withdrawal, not a harvest-quality defect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PELVIC  —  SH floor (left)  vs  ATM receipt (right)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH: parts 666541/666506/666518 · 1392 inspected, 104 fails   |   ATM: material 666541 · 512 scrapped in 2026, 555 all-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH issue category</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Units</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% of SH fails</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATM code · reason</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All-time</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% all-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Urethra / bladder damage</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>0.3365</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9972 · Laceration/Cut</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>269</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>278</v>
+      </c>
+      <c r="L7" s="15" t="n">
+        <v>0.5009</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Other / unspecified</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>0.1731</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9973 · Out of Spec</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>107</v>
+      </c>
+      <c r="L8" s="15" t="n">
+        <v>0.1928</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Short block / mesentery length</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>0.1635</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9987 · Blood Clots</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="L9" s="15" t="n">
+        <v>0.0721</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bowel damage / separation</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>0.1346</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9983 · Incorrect Dimensions</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="L10" s="15" t="n">
+        <v>0.0649</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Membrane damage</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>0.1058</v>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9986 · Bladder Length</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="L11" s="15" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical-area laceration</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>0.0577</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9995 · Received Damage</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <v>0.0378</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ureter damage</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>0.0288</v>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9988 · Exposed Urethra</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="L13" s="15" t="n">
+        <v>0.0324</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9991 · R&amp;D/Testing*</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>0.018</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9976 · Spoilage</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <v>0.0126</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1220 · Destructive Testing (eng/R&amp;D)*</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>0.0126</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9994 · Line Clearance*</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <v>0.0108</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total SH issues</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total ATM scrapped</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>512</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— quality defects only (excl. *)</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>489</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alignment: ATM's #1 code 9972 Laceration/Cut (52% of 2026 scrap) is the downstream face of the SH urethra/bladder + membrane/ureter cut damage (55 of 104 SH fails). Exposed Urethra (9988) and Bladder Length (9986) map to the same SH themes; Blood Clots (9987, 40 units) and Received Damage (9995) are ATM-only finds the floor can't see pre-freeze.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">THORACIC  —  SH floor (left)  vs  ATM receipt (right)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH: part 666521 · 76 inspected, 62 fails   |   ATM: material 666521 · 589 scrapped in 2026, 1155 all-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH issue category</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Units</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% of SH fails</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATM code · reason</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All-time</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% all-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lung laceration</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9972 · Laceration/Cut</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>384</v>
+      </c>
+      <c r="K25" s="6" t="n">
+        <v>537</v>
+      </c>
+      <c r="L25" s="15" t="n">
+        <v>0.4649</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heart damage</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>0.3333</v>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1220 · Destructive Testing (eng/R&amp;D)*</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>330</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <v>0.2857</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 · (unmapped legacy code)</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>162</v>
+      </c>
+      <c r="L27" s="15" t="n">
+        <v>0.1403</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9985 · Tech Damaged</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="L28" s="15" t="n">
+        <v>0.0424</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 · (unmapped legacy code)</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="L29" s="15" t="n">
+        <v>0.0242</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7 · Others</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K30" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <v>0.0182</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9973 · Out of Spec</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="L31" s="15" t="n">
+        <v>0.0121</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1201 · Tech Performance</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L32" s="15" t="n">
+        <v>0.0104</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 · (unmapped legacy code)</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="15" t="n">
+        <v>0.0009</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9984 · Partial Qty</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>0.0009</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total SH issues</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total ATM scrapped</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="n">
+        <v>589</v>
+      </c>
+      <c r="K35" s="6" t="n">
+        <v>1155</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— quality defects only (excl. *)</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>434</v>
+      </c>
+      <c r="K36" s="6" t="n">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alignment: both stages tell one story — lacerations. SH logs lung laceration (42) + heart damage (21); ATM 2026 scrap is 65% 9972 Laceration/Cut (384 units) plus Tech Damaged (9985). Excluding destructive testing (1220), 2026 thoracic quality scrap is 434 units on 869 received — ~50% — confirming the harvesting-side crisis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="44" customHeight="1">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Windows differ by design: SH inspections began Apr 2026 (thoracic: Jul 2026); ATM history covers Jan 2026+ for pelvic 666541 and Jul 2024+ for thoracic. The ATM '2026' column is the fairer comparison to the SH program.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="44" customHeight="1">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Category systems differ: SH categories are analyst-coded from free-text scrap notes; ATM reasons are SAP codes chosen by the reviewing tech. They describe the same physical defects at different stages — the pairing in the reads is directional, not a formal crosswalk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="44" customHeight="1">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Planned/process withdrawals marked *: 1220 Destructive Testing (eng/R&amp;D use), 9991 R&amp;D/Testing, 9994 Line Clearance. Code 7 = Others, 1201 = Tech Performance (per Quality). Legacy codes 4/5/1 (2024–25 thoracic) remain unmapped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="44" customHeight="1">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Coverage: ATM tracks only 666541 (pelvic) and 666521 (thoracic) — SH parts 666506 (non-intact) and Parks 666518 have no ATM counterpart. SH counts are floor samples; ATM counts are full received quantities.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="53">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="A37:L37"/>
+    <mergeCell ref="A39:L39"/>
+    <mergeCell ref="A40:L40"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A42:L42"/>
+    <mergeCell ref="A43:L43"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D7:D17">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K7:K17">
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFE8A33D"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D25:D34">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K25:K34">
+    <cfRule type="dataBar" priority="4">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFE8A33D"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Distinguish Nahunta two-stage tally format in the Inspection Log
Nahunta sheets from 08/26 use a two-stage tally (SH tech screens, then QC tech
inspects) unlike the standard single-stage format elsewhere. Made the
distinction explicit:
- New 'Tally format' column on the Inspection Log (Standard vs Two-stage);
  the log continues to record the FINAL QC outcome so rows stay comparable
- New 'Nahunta Two-Stage Tally - Stage Detail' section: received, SH-tech
  pass/yield (50% on 8/26, 10.5% on 9/9), QC accept of SH-passed (88.9%, 100%),
  final FPY, and stage notes, with definitions
- Note 27 documents the convention and reads the SH-tech screen as a leading
  indicator of harvesting quality
Downstream formulas (dashboard/monthly ranges, CF, freeze) unchanged and
verified. README updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/SH_IQC_Inspections.xlsx
+++ b/QC inspections suppliers/SH_IQC_Inspections.xlsx
@@ -2320,7 +2320,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M107"/>
+  <dimension ref="A1:N114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2334,6 +2334,7 @@
     <col min="9" max="11" width="9" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="55" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2343,10 +2344,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="44" customHeight="1">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Post-harvest, pre-freeze inspections at the slaughterhouse — all tissue types and parts. 65 part-inspections across 44 visit-days · 3 slaughterhouses (Martins, Parks, Nahunta) · Apr 13 – Sep 9, 2026. One row per part per harvest date.</t>
+          <t xml:space="preserve">Post-harvest, pre-freeze inspections at the slaughterhouse — all tissue types and parts. 65 part-inspections across 44 visit-days · 3 slaughterhouses (Martins, Parks, Nahunta) · Apr 13 – Sep 9, 2026. One row per part per harvest date. Two tally formats are in use (see the Tally Format column): Standard (one pass/fail count) and, at Nahunta from 08/26, Two-stage (SH tech screens, then the QC tech inspects) — the log always records the FINAL QC outcome, so rows are comparable across formats; stage detail is in the section below.</t>
         </is>
       </c>
     </row>
@@ -2424,6 +2425,11 @@
           <t xml:space="preserve">Scrap reason / notes</t>
         </is>
       </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tally format</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="27.0" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -2483,6 +2489,11 @@
           <t xml:space="preserve">3 labels used for thin area in bowel (ran out of labels)</t>
         </is>
       </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="27.0" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -2542,6 +2553,11 @@
           <t xml:space="preserve">1 hole in bowel; 1 label marked for thin area in bowel</t>
         </is>
       </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="13.5" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -2601,6 +2617,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="27.0" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -2660,6 +2681,11 @@
           <t xml:space="preserve">2 blood clots (moved to non-intact); 2 scrapped for cut in urethra</t>
         </is>
       </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="13.5" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -2719,6 +2745,11 @@
           <t xml:space="preserve">2 damaged after cleaning</t>
         </is>
       </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="27.0" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -2778,6 +2809,11 @@
           <t xml:space="preserve">Ran out of time (bagging set for later; SH tech start time changed to 8:00–4:30 PM)</t>
         </is>
       </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="13.5" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -2837,6 +2873,11 @@
           <t xml:space="preserve">2 damaged bowel</t>
         </is>
       </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="13.5" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -2896,6 +2937,11 @@
           <t xml:space="preserve">1 damaged bowel</t>
         </is>
       </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="13.5" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -2955,6 +3001,11 @@
           <t xml:space="preserve">3 damaged urethra</t>
         </is>
       </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="13.5" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -3014,6 +3065,11 @@
           <t xml:space="preserve">1 damaged urethra</t>
         </is>
       </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="13.5" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -3073,6 +3129,11 @@
           <t xml:space="preserve">1 small bladder</t>
         </is>
       </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="13.5" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -3132,6 +3193,11 @@
           <t xml:space="preserve">3 damaged urethra</t>
         </is>
       </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="13.5" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -3191,6 +3257,11 @@
           <t xml:space="preserve">1 deformed ligaments clumped together</t>
         </is>
       </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="13.5" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -3250,6 +3321,11 @@
           <t xml:space="preserve">3 cut urethra; 1 short block</t>
         </is>
       </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="13.5" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -3309,6 +3385,11 @@
           <t xml:space="preserve">1 damaged membrane and ureter</t>
         </is>
       </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="13.5" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -3368,6 +3449,11 @@
           <t xml:space="preserve">2 cut urethra</t>
         </is>
       </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="13.5" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -3427,6 +3513,11 @@
           <t xml:space="preserve">1 hole in bowel; 2 membrane damage &gt;0.5"</t>
         </is>
       </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="27.0" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -3486,6 +3577,11 @@
           <t xml:space="preserve">4 mesentery length too short in critical zone; 1 bladder damage (internals exposed)</t>
         </is>
       </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="13.5" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -3545,6 +3641,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="13.5" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -3604,6 +3705,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="13.5" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -3663,6 +3769,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="13.5" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -3722,6 +3833,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="13.5" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -3781,6 +3897,11 @@
           <t xml:space="preserve">2 scrapped urethra</t>
         </is>
       </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="13.5" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -3840,6 +3961,11 @@
           <t xml:space="preserve">1 short block</t>
         </is>
       </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="13.5" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -3899,6 +4025,11 @@
           <t xml:space="preserve">1 cut urethra</t>
         </is>
       </c>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="27.0" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -3958,6 +4089,11 @@
           <t xml:space="preserve">1 damaged bowel (source had two intact tally lines: 13/12/1 + 18/18/0, combined here)</t>
         </is>
       </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="27.0" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -4017,6 +4153,11 @@
           <t xml:space="preserve">1 bladder hole; 1 ureter damage (many blocks failed upstream from miscuts during removal — see notes)</t>
         </is>
       </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="27.0" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -4076,6 +4217,11 @@
           <t xml:space="preserve">1 bladder hole; 2 critical-area lacerations; 2 short blocks</t>
         </is>
       </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="13.5" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -4135,6 +4281,11 @@
           <t xml:space="preserve">1 damaged bladder; 3 damaged membrane</t>
         </is>
       </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="13.5" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -4194,6 +4345,11 @@
           <t xml:space="preserve">1 bladder hole; 1 ureter laceration; 1 short block</t>
         </is>
       </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="13.5" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -4253,6 +4409,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="40.0" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -4312,6 +4473,11 @@
           <t xml:space="preserve">2 damaged during bowel cleaning (bowel blockage burst); 2 short blocks; 1 critical-area laceration; 7 urethra/bladder lacerations (cuts near template edge)</t>
         </is>
       </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="13.5" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -4371,6 +4537,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="13.5" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -4430,6 +4601,11 @@
           <t xml:space="preserve">1 membrane damage larger than 1.5"</t>
         </is>
       </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="13.5" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -4489,6 +4665,11 @@
           <t xml:space="preserve">1 damaged urethra</t>
         </is>
       </c>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="13.5" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -4548,6 +4729,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="27.0" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -4607,6 +4793,11 @@
           <t xml:space="preserve">2 damaged during bowel cleaning (bowel blockage burst); 3 short blocks (smaller pigs)</t>
         </is>
       </c>
+      <c r="N42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="13.5" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -4666,6 +4857,11 @@
           <t xml:space="preserve">1 damaged membrane; 1 damaged bladder</t>
         </is>
       </c>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="27.0" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
@@ -4725,6 +4921,11 @@
           <t xml:space="preserve">2 short (bowel snapped before cut to length); 2 holes in mesentery critical area</t>
         </is>
       </c>
+      <c r="N44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="13.5" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -4784,6 +4985,11 @@
           <t xml:space="preserve">1 large membrane damage</t>
         </is>
       </c>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="40.0" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -4843,6 +5049,11 @@
           <t xml:space="preserve">1 deformed bladder documented; source #Fail cell read 1, but 65 inspected − 63 pass = 2 → 1 reject undocumented (confirm)</t>
         </is>
       </c>
+      <c r="N46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="13.5" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
@@ -4902,6 +5113,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="27.0" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -4961,6 +5177,11 @@
           <t xml:space="preserve">1 ureter damage; 1 mesentery hole in critical area &gt;0.5"; 1 bowel-colon separation past critical area</t>
         </is>
       </c>
+      <c r="N48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="13.5" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
@@ -5020,6 +5241,11 @@
           <t xml:space="preserve">1 damaged membrane larger than 0.5"</t>
         </is>
       </c>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="54.0" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
@@ -5079,6 +5305,11 @@
           <t xml:space="preserve">11 right-lung lacerations (mostly along the perimeter); 2 heart damage; 1 accepted with two sub-4cm perimeter lacerations that did not connect. Majority of damage attributed to the harvesting side.</t>
         </is>
       </c>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="13.5" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
@@ -5138,6 +5369,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="27.0" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
@@ -5197,6 +5433,11 @@
           <t xml:space="preserve">1 pelvic block short (majority of pigs received were male → lower numbers)</t>
         </is>
       </c>
+      <c r="N52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="13.5" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
@@ -5256,6 +5497,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="54.0" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
@@ -5315,6 +5561,11 @@
           <t xml:space="preserve">11 right-lung lacerations (mostly along perimeter); 4 heart damage. Majority of damage harvesting-side; two units had no lung laceration but failed on heart.</t>
         </is>
       </c>
+      <c r="N54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="13.5" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
@@ -5374,6 +5625,11 @@
           <t xml:space="preserve">1 damaged membrane; 1 hole in bowel</t>
         </is>
       </c>
+      <c r="N55" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="13.5" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
@@ -5433,6 +5689,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N56" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="13.5" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
@@ -5492,6 +5753,11 @@
           <t xml:space="preserve">2 urethra damage</t>
         </is>
       </c>
+      <c r="N57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="13.5" customHeight="1">
       <c r="A58" s="5" t="inlineStr">
@@ -5551,6 +5817,11 @@
           <t xml:space="preserve">No failures this day.</t>
         </is>
       </c>
+      <c r="N58" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="40.0" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
@@ -5610,6 +5881,11 @@
           <t xml:space="preserve">9 right-lung lacerations; 3 heart damage (breakdown sums to 12 vs 11 recorded). No left-lung damage seen; requested Ricardo shadow next visit.</t>
         </is>
       </c>
+      <c r="N59" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="40.0" customHeight="1">
       <c r="A60" s="5" t="inlineStr">
@@ -5669,6 +5945,11 @@
           <t xml:space="preserve">Pelvic deprioritized — Jordan harvests other components first; no per-defect breakdown recorded (PROVISIONAL — confirm)</t>
         </is>
       </c>
+      <c r="N60" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="27.0" customHeight="1">
       <c r="A61" s="5" t="inlineStr">
@@ -5728,6 +6009,11 @@
           <t xml:space="preserve">Bowel separated from mesentery past the critical point</t>
         </is>
       </c>
+      <c r="N61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="13.5" customHeight="1">
       <c r="A62" s="5" t="inlineStr">
@@ -5787,6 +6073,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N62" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="27.0" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
@@ -5846,6 +6137,11 @@
           <t xml:space="preserve">1 hole in bowel (ran out of pigs, 3-hr wait, truck late)</t>
         </is>
       </c>
+      <c r="N63" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="54.0" customHeight="1">
       <c r="A64" s="5" t="inlineStr">
@@ -5905,6 +6201,11 @@
           <t xml:space="preserve">11 right-lung lacerations; 12 heart damage. Ricardo meeting reduced lung lacerations only until first break; heart lacerations (inspector-side) now the next gap.</t>
         </is>
       </c>
+      <c r="N64" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="13.5" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
@@ -5964,6 +6265,11 @@
           <t xml:space="preserve">1 hole in the mesentery critical area</t>
         </is>
       </c>
+      <c r="N65" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="13.5" customHeight="1">
       <c r="A66" s="5" t="inlineStr">
@@ -6023,6 +6329,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N66" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="13.5" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
@@ -6082,6 +6393,11 @@
           <t xml:space="preserve">1 cut urethra; 1 short membrane on right side</t>
         </is>
       </c>
+      <c r="N67" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="54.0" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
@@ -6141,6 +6457,11 @@
           <t xml:space="preserve">8 lung lacerations; 2 heart lacerations. New two-stage tally: SH tech passed 9/18, QC passed 8 — incl. 2 upper-vessel-damage blocks passed &amp; labeled for a usability study. Sharp rebound after Francisco's team engagement.</t>
         </is>
       </c>
+      <c r="N68" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two-stage (SH tech → QC)</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="27.0" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
@@ -6200,6 +6521,11 @@
           <t xml:space="preserve">1 damaged membrane (SH finished early; 2.5-hr truck wait)</t>
         </is>
       </c>
+      <c r="N69" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="54.0" customHeight="1">
       <c r="A70" s="5" t="inlineStr">
@@ -6257,6 +6583,11 @@
       <c r="M70" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">8 left-lung lacerations; 9 missing trachea — SH harvesting tracheas for another buyer (low thoracic volume). One passed unit had a high head-vessel laceration, labeled.</t>
+        </is>
+      </c>
+      <c r="N70" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two-stage (SH tech → QC)</t>
         </is>
       </c>
     </row>
@@ -6356,372 +6687,541 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">NAHUNTA TWO-STAGE TALLY — STAGE DETAIL (format in use since 08/26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="27" customHeight="1">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harvest Date</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lot</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Part #</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Received</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH-Tech Pass</t>
+        </is>
+      </c>
+      <c r="F79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH-Tech Yield</t>
+        </is>
+      </c>
+      <c r="G79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC Final Pass</t>
+        </is>
+      </c>
+      <c r="H79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC Accept of SH-Passed</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Final FPY</t>
+        </is>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502539375</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666521</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F80" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G80" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8 / 9  (88.9%)</t>
+        </is>
+      </c>
+      <c r="I80" s="15" t="n">
+        <v>0.4444</v>
+      </c>
+      <c r="J80" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH tech screened 18 → 9; QC confirmed 8 (2 upper-vessel-damage blocks passed &amp; labeled for the usability study). Rebound credited to Francisco's team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502550281</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666521</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" s="15" t="n">
+        <v>0.1053</v>
+      </c>
+      <c r="G81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 / 2  (100%)</t>
+        </is>
+      </c>
+      <c r="I81" s="15" t="n">
+        <v>0.1053</v>
+      </c>
+      <c r="J81" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH tech screened 19 → 2; QC confirmed both. Fails: 8 left-lung lacerations + 9 missing trachea (SH harvesting tracheas for another buyer). One passed unit labeled for a high head-vessel laceration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="44" customHeight="1">
+      <c r="A82" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Definitions — SH-Tech Yield: blocks the slaughterhouse's own tech passed ÷ received (the sheet's “FPY for SH”). QC Accept of SH-Passed: of the SH-tech-passed blocks, how many our QC tech confirmed (the sheet's “FPY for SH Tech”). Final FPY = QC final pass ÷ received — this is the number carried into the Inspection Log, dashboards and monthly tabs, so all cross-site comparisons remain final-outcome to final-outcome. Nahunta visits before 08/26 (7/29, 8/5, 8/12, 8/19) used the Standard single-stage tally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83"/>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">ATM RECEIPT COMPARISON</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="30" customHeight="1">
-      <c r="A79" s="20" t="inlineStr">
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">See the 'SH vs ATM by Batch' and 'SH vs ATM Issues' tabs. The current ATM (SAP) extract runs through 09/16 — batches harvested after that will appear in the comparison when the next extract arrives.</t>
         </is>
       </c>
     </row>
-    <row r="80"/>
-    <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="3" t="inlineStr">
+    <row r="86"/>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">NOTES &amp; DATA CONVENTIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="60.0" customHeight="1">
-      <c r="A82" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. 666506 = non-intact</t>
-        </is>
-      </c>
-      <c r="B82" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In the source tally sheets, PN 666541 is labeled 'intact' and PN 666506 is labeled 'Non intact'. Scrap reasons include phrases like '2 blood clots, moved to non intact', suggesting 666506 is a downgrade/recovery spec rather than an independent product line. Confirm with Quality before relying on this interpretation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="60.0" customHeight="1">
-      <c r="A83" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2. Different lot suffixes for intact vs non-intact</t>
-        </is>
-      </c>
-      <c r="B83" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Intact and non-intact batches from the same kill day carry DIFFERENT lot numbers (e.g. Visit 1: 5502378434 intact / 5502378430 non-intact; Visit 3: 5502404928 intact / 5502404924 non-intact). The prefix ties them to the same kill but they are tracked separately. This is what 'same batch number but not exactly' refers to.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="60.0" customHeight="1">
-      <c r="A84" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3. 'Ran out of time' event on 04/20</t>
-        </is>
-      </c>
-      <c r="B84" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lot 5502391862 intact had zero units inspected on 04/20 due to a schedule conflict (bagging set later, SH tech start time changed to 8:00–4:30 PM). 57 units from that lot were inspected on 04/22 instead. Process note, not a quality signal — but if it recurs, sampling discipline at the slaughterhouse is worth revisiting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="60.0" customHeight="1">
-      <c r="A85" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4. 'Damaged urethra' dominates Visit 3</t>
-        </is>
-      </c>
-      <c r="B85" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On Visit 3 (05/04 + 05/06), 7 of 8 failures across both intact and non-intact were 'damaged urethra' — a sharp departure from prior visits, where bowel-related defects dominated. Worth checking whether harvest technique or tooling changed, or whether the long pre-inspection wait on 05/04 (see next note) contributed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="60.0" customHeight="1">
-      <c r="A86" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5. Long truck wait on 05/04 (Visit 3)</t>
-        </is>
-      </c>
-      <c r="B86" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Source tally-sheet notes record: 'Monday 05/04 waited 2 hour for truck to deliver at 10:15 am. Had almost 3 hours of waiting.' Tissue sitting longer pre-inspection plausibly correlates with the urethra-damage spike that day. Worth tagging future inspections with delivery time so this can be analyzed quantitatively.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="60.0" customHeight="1">
-      <c r="A87" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6. Source file typos</t>
-        </is>
-      </c>
-      <c r="B87" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Source tally sheets carry '25026' instead of '2026' in the Date and Kill Date fields (Harvest Date is correct). Not reflected here — clean dates used throughout. One-line correction in the tally-sheet template would fix it going forward.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="60.0" customHeight="1">
       <c r="A88" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">7. Stage-to-stage scope</t>
+          <t xml:space="preserve">1. 666506 = non-intact</t>
         </is>
       </c>
       <c r="B88" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Three lots now have BOTH SH and ATM data: 5502378434, 5502391862, and 5502404928. The 666506 non-intact lots remain untracked at ATM. As lots accumulate, the SH-vs-ATM yield gap is the cleanest available proxy for freeze/thaw/transport damage.</t>
+          <t xml:space="preserve">In the source tally sheets, PN 666541 is labeled 'intact' and PN 666506 is labeled 'Non intact'. Scrap reasons include phrases like '2 blood clots, moved to non intact', suggesting 666506 is a downgrade/recovery spec rather than an independent product line. Confirm with Quality before relying on this interpretation.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="60.0" customHeight="1">
       <c r="A89" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">8. Inspection coverage</t>
+          <t xml:space="preserve">2. Different lot suffixes for intact vs non-intact</t>
         </is>
       </c>
       <c r="B89" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">65 part-inspections across 44 visit-days and 3 slaughterhouses (Martins ×25, Parks ×13, Nahunta ×6), Apr 13 – Sep 9 2026. Tissue types: Pelvic (666541/666506/666518) and Thoracic (666521). To extend, append rows to the log; the SUMIF/SUM ranges auto-cover them.</t>
+          <t xml:space="preserve">Intact and non-intact batches from the same kill day carry DIFFERENT lot numbers (e.g. Visit 1: 5502378434 intact / 5502378430 non-intact; Visit 3: 5502404928 intact / 5502404924 non-intact). The prefix ties them to the same kill but they are tracked separately. This is what 'same batch number but not exactly' refers to.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="60.0" customHeight="1">
       <c r="A90" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">9. Lot 5502421192 reused on the 05/27 sheet</t>
+          <t xml:space="preserve">3. 'Ran out of time' event on 04/20</t>
         </is>
       </c>
       <c r="B90" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">The 05/27 Martins tally sheet records the intact lot as 5502421192 — identical to Visit 4's intact lot (harvested 05/18 &amp; 05/21). A single fresh lot spanning 05/18–05/27 is unlikely, so this is probably a tally-sheet carry-over from the prior week's template. It is recorded here as a separate Visit 5 (harvest 05/27), NOT merged into Visit 4, pending confirmation of the true lot number with the SH.</t>
+          <t xml:space="preserve">Lot 5502391862 intact had zero units inspected on 04/20 due to a schedule conflict (bagging set later, SH tech start time changed to 8:00–4:30 PM). 57 units from that lot were inspected on 04/22 instead. Process note, not a quality signal — but if it recurs, sampling discipline at the slaughterhouse is worth revisiting.</t>
         </is>
       </c>
     </row>
     <row r="91" ht="60.0" customHeight="1">
       <c r="A91" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">10. New slaughterhouse &amp; inspection team (Parks, 05/28)</t>
+          <t xml:space="preserve">4. 'Damaged urethra' dominates Visit 3</t>
         </is>
       </c>
       <c r="B91" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">First SH-floor inspection at Parks Family Meats, with a new ATM inspector (Rasmin) and new SH tech (Natalie) vs. Toni / Jesus at Martins. Source PN was written 668518 and normalized to 666518 (per the workbook's typo convention). No batch/lot was recorded ('no batch data'), so this visit has no SH→ATM link, and the related Parks ATM lot 5502428883 (7 received / 7 scrapped, 'before our visit') has no SH-floor counterpart here. Date taken from the source date field (05/28); the carried-over note text mentioning '5/27' and non-intact labels does not apply to this intact-only Parks visit.</t>
+          <t xml:space="preserve">On Visit 3 (05/04 + 05/06), 7 of 8 failures across both intact and non-intact were 'damaged urethra' — a sharp departure from prior visits, where bowel-related defects dominated. Worth checking whether harvest technique or tooling changed, or whether the long pre-inspection wait on 05/04 (see next note) contributed.</t>
         </is>
       </c>
     </row>
     <row r="92" ht="60.0" customHeight="1">
       <c r="A92" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">11. Visit 7 harvest-date split (06/01 vs 06/03)</t>
+          <t xml:space="preserve">5. Long truck wait on 05/04 (Visit 3)</t>
         </is>
       </c>
       <c r="B92" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">The 06/01 &amp; 06/03 Martins tally sheet did not label which counts belong to which day. Based on the note that 06/01 finished early (truck no-show, cleanup 1pm), the smaller counts were assigned to 06/01 (9 intact, 7 non-intact) and the larger to 06/03 (45 intact, 29 non-intact), placing the 2 urethra scraps on 06/03. Flip the two raw rows if the source intended otherwise — the batch-level rollup is identical either way.</t>
+          <t xml:space="preserve">Source tally-sheet notes record: 'Monday 05/04 waited 2 hour for truck to deliver at 10:15 am. Had almost 3 hours of waiting.' Tissue sitting longer pre-inspection plausibly correlates with the urethra-damage spike that day. Worth tagging future inspections with delivery time so this can be analyzed quantitatively.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="60.0" customHeight="1">
       <c r="A93" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">12. New visits 7 (Martins) &amp; 8 (Parks)</t>
+          <t xml:space="preserve">6. Source file typos</t>
         </is>
       </c>
       <c r="B93" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visit 7 adds intact lot 5502428786 and non-intact lot 5502428782 (Martins). Visit 8 is the second Parks visit (intact-only, no batch/lot; PN normalized 668518 → 666518). The Parks visit date 06/02 is the cached value of a volatile =NOW()-1 field on the source sheet, so it is nominal. One non-intact Martins row (29 inspected) had a blank pass cell on the source; recorded as 29 pass since fail = 0.</t>
+          <t xml:space="preserve">Source tally sheets carry '25026' instead of '2026' in the Date and Kill Date fields (Harvest Date is correct). Not reflected here — clean dates used throughout. One-line correction in the tally-sheet template would fix it going forward.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="60.0" customHeight="1">
       <c r="A94" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">13. New visits 9–12 (06/08–06/24)</t>
+          <t xml:space="preserve">7. Stage-to-stage scope</t>
         </is>
       </c>
       <c r="B94" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visit 9 = 06/08 Martins; Visit 10 = 06/15 Martins; Visit 11 = 06/16 Parks (intact-only); Visit 12 = 06/24 Martins (intact-only). Source date/kill fields on several incoming sheets are volatile =NOW() captures (e.g. the Parks sheet sent 06/17 reads 06/16); the hand-entered harvest-date fields were used as the authoritative visit dates.</t>
+          <t xml:space="preserve">Three lots now have BOTH SH and ATM data: 5502378434, 5502391862, and 5502404928. The 666506 non-intact lots remain untracked at ATM. As lots accumulate, the SH-vs-ATM yield gap is the cleanest available proxy for freeze/thaw/transport damage.</t>
         </is>
       </c>
     </row>
     <row r="95" ht="60.0" customHeight="1">
       <c r="A95" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">14. Lot-number carry-over recurs (Visits 9 &amp; 12)</t>
+          <t xml:space="preserve">8. Inspection coverage</t>
         </is>
       </c>
       <c r="B95" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visit 9 (06/08) reuses Visit 7’s lots 5502428786/5502428782, and Visit 12 (06/24) reuses Visit 10’s intact lot 5502462845 — the same template carry-over pattern documented in note 9 for lot 5502421192. Each is recorded as its own visit with its own raw and rollup rows, but per the note-9 precedent only the FIRST occurrence of each lot is reconciled in the SH→ATM section, so the reused-lot inspections do not generate duplicate SH→ATM rows.</t>
+          <t xml:space="preserve">65 part-inspections across 44 visit-days and 3 slaughterhouses (Martins ×25, Parks ×13, Nahunta ×6), Apr 13 – Sep 9 2026. Tissue types: Pelvic (666541/666506/666518) and Thoracic (666521). To extend, append rows to the log; the SUMIF/SUM ranges auto-cover them.</t>
         </is>
       </c>
     </row>
     <row r="96" ht="60.0" customHeight="1">
       <c r="A96" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">15. Visit 10 (06/15) — two intact tally lines combined; no non-intact</t>
+          <t xml:space="preserve">9. Lot 5502421192 reused on the 05/27 sheet</t>
         </is>
       </c>
       <c r="B96" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">The source recorded two intact 666541 lines on 06/15 (13/12/1 and 18/18/0); they share date, lot and condition, so they are combined into a single raw row (31/30/1). No non-intact units were collected (the SH had met its non-intact quota and run low on labels), so lot 5502462842 appears in the metadata but has no raw/rollup row.</t>
+          <t xml:space="preserve">The 05/27 Martins tally sheet records the intact lot as 5502421192 — identical to Visit 4's intact lot (harvested 05/18 &amp; 05/21). A single fresh lot spanning 05/18–05/27 is unlikely, so this is probably a tally-sheet carry-over from the prior week's template. It is recorded here as a separate Visit 5 (harvest 05/27), NOT merged into Visit 4, pending confirmation of the true lot number with the SH.</t>
         </is>
       </c>
     </row>
     <row r="97" ht="60.0" customHeight="1">
       <c r="A97" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">16. Visit 11 (06/16 Parks) — heavy upstream miscut losses</t>
+          <t xml:space="preserve">10. New slaughterhouse &amp; inspection team (Parks, 05/28)</t>
         </is>
       </c>
       <c r="B97" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">The inspector noted ~100 pigs slaughtered, with the majority of blocks failing BEFORE reaching IQC due to miscuts during block removal. Of the 16 that reached inspection, 14 passed (1 bladder hole, 1 ureter damage). That upstream loss is a Parks harvest-technique signal not captured in the pass/fail counts here. PN normalized 668518 → 666518 per note 10. Separately, the “PARKS0603” sheet (internal date 06/02, 7/7 intact, no batch) is the SAME inspection already recorded as Visit 8 and was not re-added.</t>
+          <t xml:space="preserve">First SH-floor inspection at Parks Family Meats, with a new ATM inspector (Rasmin) and new SH tech (Natalie) vs. Toni / Jesus at Martins. Source PN was written 668518 and normalized to 666518 (per the workbook's typo convention). No batch/lot was recorded ('no batch data'), so this visit has no SH→ATM link, and the related Parks ATM lot 5502428883 (7 received / 7 scrapped, 'before our visit') has no SH-floor counterpart here. Date taken from the source date field (05/28); the carried-over note text mentioning '5/27' and non-intact labels does not apply to this intact-only Parks visit.</t>
         </is>
       </c>
     </row>
     <row r="98" ht="60.0" customHeight="1">
       <c r="A98" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">17. New Parks visits 13 (06/22) &amp; 14 (06/25)</t>
+          <t xml:space="preserve">11. Visit 7 harvest-date split (06/01 vs 06/03)</t>
         </is>
       </c>
       <c r="B98" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two more intact-only Parks inspections (no batch data; PN normalized 668518 → 666518). Visit 13 (06/22) = 36 inspected / 31 pass / 5 fail (1 bladder hole, 2 critical-area lacerations, 2 short blocks); Visit 14 (06/25) = 19 inspected / 16 pass / 3 fail (1 bladder hole, 1 ureter laceration, 1 short block). Both were received after Visit 12, so Visit 13’s harvest date (06/22) precedes Visit 12’s (06/24 Martins) — visit numbers reflect processing order, as with the existing Visit 7/8 overlap. No batch on either, so neither has an SH→ATM link (consistent with Visits 6, 8 and 11). Short blocks and critical-zone mesentery damage continue to dominate Parks scrap.</t>
+          <t xml:space="preserve">The 06/01 &amp; 06/03 Martins tally sheet did not label which counts belong to which day. Based on the note that 06/01 finished early (truck no-show, cleanup 1pm), the smaller counts were assigned to 06/01 (9 intact, 7 non-intact) and the larger to 06/03 (45 intact, 29 non-intact), placing the 2 urethra scraps on 06/03. Flip the two raw rows if the source intended otherwise — the batch-level rollup is identical either way.</t>
         </is>
       </c>
     </row>
     <row r="99" ht="60.0" customHeight="1">
       <c r="A99" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">18. New visits 15–19 (06/29–07/13); two Parks fail-count corrections</t>
+          <t xml:space="preserve">12. New visits 7 (Martins) &amp; 8 (Parks)</t>
         </is>
       </c>
       <c r="B99" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visit 15 = 06/29 Martins; Visit 16 = 06/29 Parks; Visit 17 = 07/06 Martins; Visit 18 = 07/13 Martins; Visit 19 = 07/13 Parks. DATA-ACCURACY FIX: on both Parks sheets the source “# Fail” cell undercounted because blocks damaged during bowel-cleaning were written in the notes but not added to the fail tally. Corrected to inspected − pass, which matches the scrap breakdown — Visit 16 (06/29) = 50/38/12 (source cell read 10; 2 cleaning-damage + 2 short + 1 critical + 7 urethra/bladder = 12); Visit 19 (07/13) = 34/29/5 (source cell read 3; 2 cleaning-damage + 3 short = 5). Visit 17 (07/06) reuses Visit 15’s lots 5502471460/5502471457 — a tally-sheet carry-over recorded as a separate visit (see note 9). Visit 18’s inspector field was blank on the source; recorded as Toni, the standing Martins inspector.</t>
+          <t xml:space="preserve">Visit 7 adds intact lot 5502428786 and non-intact lot 5502428782 (Martins). Visit 8 is the second Parks visit (intact-only, no batch/lot; PN normalized 668518 → 666518). The Parks visit date 06/02 is the cached value of a volatile =NOW()-1 field on the source sheet, so it is nominal. One non-intact Martins row (29 inspected) had a blank pass cell on the source; recorded as 29 pass since fail = 0.</t>
         </is>
       </c>
     </row>
     <row r="100" ht="60.0" customHeight="1">
       <c r="A100" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">19. Visit 19 (Parks) harvest-date ambiguity</t>
+          <t xml:space="preserve">13. New visits 9–12 (06/08–06/24)</t>
         </is>
       </c>
       <c r="B100" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">The source file is named “PARKS_0713” (→ 07/13), was sent as a most-recent inspection, and a Martins 07/13 sheet arrived in the same batch — so Visit 19 is recorded as harvest 07/13/2026. However, all three internal date fields on that sheet (Date, Kill, Harvest) read 06/13/2026, likely a month typo. If 06/13 was intended, flip Visit 19’s date; the counts (34/29/5) are unaffected either way.</t>
+          <t xml:space="preserve">Visit 9 = 06/08 Martins; Visit 10 = 06/15 Martins; Visit 11 = 06/16 Parks (intact-only); Visit 12 = 06/24 Martins (intact-only). Source date/kill fields on several incoming sheets are volatile =NOW() captures (e.g. the Parks sheet sent 06/17 reads 06/16); the hand-entered harvest-date fields were used as the authoritative visit dates.</t>
         </is>
       </c>
     </row>
     <row r="101" ht="60.0" customHeight="1">
       <c r="A101" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">20. New visits 20–23 (07/20–07/30); first thoracic &amp; new slaughterhouse</t>
+          <t xml:space="preserve">14. Lot-number carry-over recurs (Visits 9 &amp; 12)</t>
         </is>
       </c>
       <c r="B101" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visit 20 = 07/20 Martins (reuses Visit 18 lots 5502495107 / 5502495104 — carry-over); Visit 21 = 07/27 Martins (new lots 5502512228 / 5502512225); Visit 22 = 07/29 Nahunta — the first THORACIC (PN 666521, lot 5502512218), a new product family at a new slaughterhouse with a new inspector/tech (Kris / Jordan), 19 inspected / 6 pass / 13 fail (31.6%); Visit 23 = 07/30 Parks (666518, majority-male pigs noted). The thoracic is logged in the raw data and summarized on the "Quality Summary by Part" tab, but is EXCLUDED from the pelvic-block rollup, TOTAL and SH→ATM sections so pelvic yield stays comparable across a single product family.</t>
+          <t xml:space="preserve">Visit 9 (06/08) reuses Visit 7’s lots 5502428786/5502428782, and Visit 12 (06/24) reuses Visit 10’s intact lot 5502462845 — the same template carry-over pattern documented in note 9 for lot 5502421192. Each is recorded as its own visit with its own raw and rollup rows, but per the note-9 precedent only the FIRST occurrence of each lot is reconciled in the SH→ATM section, so the reused-lot inspections do not generate duplicate SH→ATM rows.</t>
         </is>
       </c>
     </row>
     <row r="102" ht="60.0" customHeight="1">
       <c r="A102" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">21. Visit 20 (07/20 Martins 666541) count discrepancy</t>
+          <t xml:space="preserve">15. Visit 10 (06/15) — two intact tally lines combined; no non-intact</t>
         </is>
       </c>
       <c r="B102" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">The source tally read 65 inspected / 63 pass / 1 fail, which does not foot (65 − 63 = 2), and only one defect (deformed bladder) was written in. Recorded here as 65 / 63 / 2 to preserve the two counted columns and the workbook’s fail = inspected − pass convention. If the true fail is 1, correct the pass to 64 (or inspected to 64) and the second reject’s reason. Confirm with the tech.</t>
+          <t xml:space="preserve">The source recorded two intact 666541 lines on 06/15 (13/12/1 and 18/18/0); they share date, lot and condition, so they are combined into a single raw row (31/30/1). No non-intact units were collected (the SH had met its non-intact quota and run low on labels), so lot 5502462842 appears in the metadata but has no raw/rollup row.</t>
         </is>
       </c>
     </row>
     <row r="103" ht="60.0" customHeight="1">
       <c r="A103" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">22. Workbook redesign</t>
+          <t xml:space="preserve">16. Visit 11 (06/16 Parks) — heavy upstream miscut losses</t>
         </is>
       </c>
       <c r="B103" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Single tissue-agnostic inspection log (all tissue types in one chronological table) with tissue-type subtotals and a grand total covering every tissue type; metrics broken out by Tissue Type, Part and Slaughterhouse on the Quality Dashboard. The ATM Tableau tab and the legacy ATM-side analysis tabs (Receipt Summary, Master Data, Defect Pivots, Supplier Comparison, Defect Trends) were removed; ATM receipt data will be re-added in a batch-less format.</t>
+          <t xml:space="preserve">The inspector noted ~100 pigs slaughtered, with the majority of blocks failing BEFORE reaching IQC due to miscuts during block removal. Of the 16 that reached inspection, 14 passed (1 bladder hole, 1 ureter damage). That upstream loss is a Parks harvest-technique signal not captured in the pass/fail counts here. PN normalized 668518 → 666518 per note 10. Separately, the “PARKS0603” sheet (internal date 06/02, 7/7 intact, no batch) is the SAME inspection already recorded as Visit 8 and was not re-added.</t>
         </is>
       </c>
     </row>
     <row r="104" ht="60.0" customHeight="1">
       <c r="A104" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">23. August batch (07/16–08/19) &amp; de-duplication</t>
+          <t xml:space="preserve">17. New Parks visits 13 (06/22) &amp; 14 (06/25)</t>
         </is>
       </c>
       <c r="B104" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added 15 new part-inspections across Martins, Parks and Nahunta. Re-sent sheets for 07/20, 07/27, 07/29 (thoracic) and 07/30 were matched to existing rows, not double-counted. Flags: Martins 08/03–08/05 lot recorded 5502512228 (source read '550251228', one digit dropped); Parks 07/16 harvest date taken from the filename/kill date (sheet Date field read 06/13 — typo); Parks 08/10 dated per filename (sheet Date field read 08/14).</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="46.0" customHeight="1">
+          <t xml:space="preserve">Two more intact-only Parks inspections (no batch data; PN normalized 668518 → 666518). Visit 13 (06/22) = 36 inspected / 31 pass / 5 fail (1 bladder hole, 2 critical-area lacerations, 2 short blocks); Visit 14 (06/25) = 19 inspected / 16 pass / 3 fail (1 bladder hole, 1 ureter laceration, 1 short block). Both were received after Visit 12, so Visit 13’s harvest date (06/22) precedes Visit 12’s (06/24 Martins) — visit numbers reflect processing order, as with the existing Visit 7/8 overlap. No batch on either, so neither has an SH→ATM link (consistent with Visits 6, 8 and 11). Short blocks and critical-zone mesentery damage continue to dominate Parks scrap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="60.0" customHeight="1">
       <c r="A105" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">24. Parks spec transition 666518 → 666541</t>
+          <t xml:space="preserve">18. New visits 15–19 (06/29–07/13); two Parks fail-count corrections</t>
         </is>
       </c>
       <c r="B105" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parks pelvic blocks are now received under PN 666541 (from 08/10); earlier Parks visits used 668518 → 666518. Both are Pelvic tissue; the by-part view now shows 666541 at Martins, Parks and Nahunta.</t>
+          <t xml:space="preserve">Visit 15 = 06/29 Martins; Visit 16 = 06/29 Parks; Visit 17 = 07/06 Martins; Visit 18 = 07/13 Martins; Visit 19 = 07/13 Parks. DATA-ACCURACY FIX: on both Parks sheets the source “# Fail” cell undercounted because blocks damaged during bowel-cleaning were written in the notes but not added to the fail tally. Corrected to inspected − pass, which matches the scrap breakdown — Visit 16 (06/29) = 50/38/12 (source cell read 10; 2 cleaning-damage + 2 short + 1 critical + 7 urethra/bladder = 12); Visit 19 (07/13) = 34/29/5 (source cell read 3; 2 cleaning-damage + 3 short = 5). Visit 17 (07/06) reuses Visit 15’s lots 5502471460/5502471457 — a tally-sheet carry-over recorded as a separate visit (see note 9). Visit 18’s inspector field was blank on the source; recorded as Toni, the standing Martins inspector.</t>
         </is>
       </c>
     </row>
     <row r="106" ht="60.0" customHeight="1">
       <c r="A106" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">25. Nahunta thoracic (666521) trend &amp; pelvic line</t>
+          <t xml:space="preserve">19. Visit 19 (Parks) harvest-date ambiguity</t>
         </is>
       </c>
       <c r="B106" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">First-pass yield fell 32% (7/29) → 0% (8/5) → 15% (8/12) → 21% (8/19); right-lung perimeter and increasingly heart lacerations dominate (harvesting-side; escalated with Ricardo). The 8/12 pelvic 666541 line reads 13/1/12 with no per-defect breakdown (pelvics deprioritized — Jordan harvests other components first); treat as provisional, confirm.</t>
+          <t xml:space="preserve">The source file is named “PARKS_0713” (→ 07/13), was sent as a most-recent inspection, and a Martins 07/13 sheet arrived in the same batch — so Visit 19 is recorded as harvest 07/13/2026. However, all three internal date fields on that sheet (Date, Kill, Harvest) read 06/13/2026, likely a month typo. If 06/13 was intended, flip Visit 19’s date; the counts (34/29/5) are unaffected either way.</t>
         </is>
       </c>
     </row>
     <row r="107" ht="60.0" customHeight="1">
       <c r="A107" s="19" t="inlineStr">
         <is>
+          <t xml:space="preserve">20. New visits 20–23 (07/20–07/30); first thoracic &amp; new slaughterhouse</t>
+        </is>
+      </c>
+      <c r="B107" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visit 20 = 07/20 Martins (reuses Visit 18 lots 5502495107 / 5502495104 — carry-over); Visit 21 = 07/27 Martins (new lots 5502512228 / 5502512225); Visit 22 = 07/29 Nahunta — the first THORACIC (PN 666521, lot 5502512218), a new product family at a new slaughterhouse with a new inspector/tech (Kris / Jordan), 19 inspected / 6 pass / 13 fail (31.6%); Visit 23 = 07/30 Parks (666518, majority-male pigs noted). The thoracic is logged in the raw data and summarized on the "Quality Summary by Part" tab, but is EXCLUDED from the pelvic-block rollup, TOTAL and SH→ATM sections so pelvic yield stays comparable across a single product family.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="60.0" customHeight="1">
+      <c r="A108" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21. Visit 20 (07/20 Martins 666541) count discrepancy</t>
+        </is>
+      </c>
+      <c r="B108" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The source tally read 65 inspected / 63 pass / 1 fail, which does not foot (65 − 63 = 2), and only one defect (deformed bladder) was written in. Recorded here as 65 / 63 / 2 to preserve the two counted columns and the workbook’s fail = inspected − pass convention. If the true fail is 1, correct the pass to 64 (or inspected to 64) and the second reject’s reason. Confirm with the tech.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="60.0" customHeight="1">
+      <c r="A109" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22. Workbook redesign</t>
+        </is>
+      </c>
+      <c r="B109" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single tissue-agnostic inspection log (all tissue types in one chronological table) with tissue-type subtotals and a grand total covering every tissue type; metrics broken out by Tissue Type, Part and Slaughterhouse on the Quality Dashboard. The ATM Tableau tab and the legacy ATM-side analysis tabs (Receipt Summary, Master Data, Defect Pivots, Supplier Comparison, Defect Trends) were removed; ATM receipt data will be re-added in a batch-less format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="60.0" customHeight="1">
+      <c r="A110" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23. August batch (07/16–08/19) &amp; de-duplication</t>
+        </is>
+      </c>
+      <c r="B110" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Added 15 new part-inspections across Martins, Parks and Nahunta. Re-sent sheets for 07/20, 07/27, 07/29 (thoracic) and 07/30 were matched to existing rows, not double-counted. Flags: Martins 08/03–08/05 lot recorded 5502512228 (source read '550251228', one digit dropped); Parks 07/16 harvest date taken from the filename/kill date (sheet Date field read 06/13 — typo); Parks 08/10 dated per filename (sheet Date field read 08/14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="46.0" customHeight="1">
+      <c r="A111" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24. Parks spec transition 666518 → 666541</t>
+        </is>
+      </c>
+      <c r="B111" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parks pelvic blocks are now received under PN 666541 (from 08/10); earlier Parks visits used 668518 → 666518. Both are Pelvic tissue; the by-part view now shows 666541 at Martins, Parks and Nahunta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="60.0" customHeight="1">
+      <c r="A112" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25. Nahunta thoracic (666521) trend &amp; pelvic line</t>
+        </is>
+      </c>
+      <c r="B112" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-pass yield fell 32% (7/29) → 0% (8/5) → 15% (8/12) → 21% (8/19); right-lung perimeter and increasingly heart lacerations dominate (harvesting-side; escalated with Ricardo). The 8/12 pelvic 666541 line reads 13/1/12 with no per-defect breakdown (pelvics deprioritized — Jordan harvests other components first); treat as provisional, confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="60.0" customHeight="1">
+      <c r="A113" s="19" t="inlineStr">
+        <is>
           <t xml:space="preserve">26. Late-Aug / Sep batch (08/20–09/09)</t>
         </is>
       </c>
-      <c r="B107" s="20" t="inlineStr">
+      <c r="B113" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">Five new sheets, no duplicates. Flags: the Parks file was named 08_21 but every date field reads 08/20 — recorded 08/20. Nahunta 8/26 lot read '55025239375' (11 digits) — recorded 5502539375. Nahunta switched to a two-stage tally (SH-tech and QC-tech pass/fail); the log records the final QC outcome with stage detail in the scrap notes. 08/31 Martins listed 666506 with 0 inspected and no non-intact lot — omitted. 9/9 introduces a new defect, MISSING TRACHEA (9 units): the SH is harvesting tracheas for another buyer. 8/26 shows a sharp thoracic rebound (44%) after Francisco's team engagement.</t>
         </is>
       </c>
     </row>
+    <row r="114" ht="60.0" customHeight="1">
+      <c r="A114" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">27. Nahunta two-stage tally format</t>
+        </is>
+      </c>
+      <c r="B114" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From 08/26, Nahunta tally sheets carry two stages: the SH tech's own screen (received / passed / failed) and our QC tech's inspection of the SH-passed blocks. The log's # Inspected / # Pass / # Fail are the FINAL QC outcome (received / QC pass / received − QC pass), keeping every row comparable across sites and formats; the per-stage numbers live in the NAHUNTA TWO-STAGE TALLY section above and the Tally Format column flags the affected rows. The SH-tech screen is a leading indicator of harvesting quality (50% on 8/26, 10.5% on 9/9); the QC-accept-of-SH-passed rate (88.9%, 100%) shows how well the SH tech's judgement aligns with our spec.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A72:M72"/>
-    <mergeCell ref="A78:M78"/>
-    <mergeCell ref="A79:M79"/>
-    <mergeCell ref="A81:M81"/>
-    <mergeCell ref="B82:M82"/>
-    <mergeCell ref="B83:M83"/>
-    <mergeCell ref="B84:M84"/>
-    <mergeCell ref="B85:M85"/>
-    <mergeCell ref="B86:M86"/>
-    <mergeCell ref="B87:M87"/>
-    <mergeCell ref="B88:M88"/>
-    <mergeCell ref="B89:M89"/>
-    <mergeCell ref="B90:M90"/>
-    <mergeCell ref="B91:M91"/>
-    <mergeCell ref="B92:M92"/>
-    <mergeCell ref="B93:M93"/>
-    <mergeCell ref="B94:M94"/>
-    <mergeCell ref="B95:M95"/>
-    <mergeCell ref="B96:M96"/>
-    <mergeCell ref="B97:M97"/>
-    <mergeCell ref="B98:M98"/>
-    <mergeCell ref="B99:M99"/>
-    <mergeCell ref="B100:M100"/>
-    <mergeCell ref="B101:M101"/>
-    <mergeCell ref="B102:M102"/>
-    <mergeCell ref="B103:M103"/>
-    <mergeCell ref="B104:M104"/>
-    <mergeCell ref="B105:M105"/>
-    <mergeCell ref="B106:M106"/>
-    <mergeCell ref="B107:M107"/>
+  <mergeCells count="39">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A72:N72"/>
+    <mergeCell ref="A78:N78"/>
+    <mergeCell ref="J79:N79"/>
+    <mergeCell ref="J80:N80"/>
+    <mergeCell ref="J81:N81"/>
+    <mergeCell ref="A82:N82"/>
+    <mergeCell ref="A84:N84"/>
+    <mergeCell ref="A85:N85"/>
+    <mergeCell ref="A87:N87"/>
+    <mergeCell ref="B88:N88"/>
+    <mergeCell ref="B89:N89"/>
+    <mergeCell ref="B90:N90"/>
+    <mergeCell ref="B91:N91"/>
+    <mergeCell ref="B92:N92"/>
+    <mergeCell ref="B93:N93"/>
+    <mergeCell ref="B94:N94"/>
+    <mergeCell ref="B95:N95"/>
+    <mergeCell ref="B96:N96"/>
+    <mergeCell ref="B97:N97"/>
+    <mergeCell ref="B98:N98"/>
+    <mergeCell ref="B99:N99"/>
+    <mergeCell ref="B100:N100"/>
+    <mergeCell ref="B101:N101"/>
+    <mergeCell ref="B102:N102"/>
+    <mergeCell ref="B103:N103"/>
+    <mergeCell ref="B104:N104"/>
+    <mergeCell ref="B105:N105"/>
+    <mergeCell ref="B106:N106"/>
+    <mergeCell ref="B107:N107"/>
+    <mergeCell ref="B108:N108"/>
+    <mergeCell ref="B109:N109"/>
+    <mergeCell ref="B110:N110"/>
+    <mergeCell ref="B111:N111"/>
+    <mergeCell ref="B112:N112"/>
+    <mergeCell ref="B113:N113"/>
+    <mergeCell ref="B114:N114"/>
   </mergeCells>
   <conditionalFormatting sqref="L6:L70">
     <cfRule type="colorScale" priority="1">

</xml_diff>

<commit_message>
Pre-receipt reframing for Nahunta 8/12 pelvic line; QC numbers lead two-stage table; deck cut to 2 slides
- The Nahunta 8/12 pelvic line (13/1/12) was inspected prior to receiving the
  tissue (before the harvesting tech got it): no longer red/FPY-graded anywhere,
  relabeled 'Pre-receipt screen', with the note on the log, dashboard, monthly,
  Aug tab, issues tab and slides. Totals unchanged.
- Two-inspection stage table now leads with the QC pass numbers (8/1 88.9%,
  2/0 100%); the notes explain what it took to get the good ones (18->9->8,
  19->2->2).
- QDR deck reduced to slides 1 and 3 per request (batch slide and two-stage
  slide removed); slide content is August SH inspections, ATM side restricted
  to SH-inspected batches.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/SH_IQC_Inspections.xlsx
+++ b/QC inspections suppliers/SH_IQC_Inspections.xlsx
@@ -6045,12 +6045,12 @@
       </c>
       <c r="M60" s="60" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNVERIFIED — no scrap reasons recorded on the source sheet (totals only). Pelvics deprioritized on the line (Jordan harvests other components from the blocks). Counts provisional; EXCLUDED from defect-profile charts pending confirmation with Kris.</t>
+          <t xml:space="preserve">PRE-RECEIPT SCREEN — these 13 blocks were inspected prior to receiving them (before the harvesting tech got the tissue); the 12 rejects never became received product, so this line is not graded as incoming first-pass yield. No scrap reasons itemized on the source sheet; excluded from defect-profile charts.</t>
         </is>
       </c>
       <c r="N60" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNVERIFIED</t>
+          <t xml:space="preserve">Pre-receipt screen</t>
         </is>
       </c>
     </row>
@@ -6819,41 +6819,41 @@
       </c>
       <c r="D80" s="53" t="inlineStr">
         <is>
+          <t xml:space="preserve">QC Pass</t>
+        </is>
+      </c>
+      <c r="E80" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC Fail</t>
+        </is>
+      </c>
+      <c r="F80" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC FPY (log basis)</t>
+        </is>
+      </c>
+      <c r="G80" s="53" t="inlineStr">
+        <is>
           <t xml:space="preserve"># Received at harvest</t>
         </is>
       </c>
-      <c r="E80" s="53" t="inlineStr">
+      <c r="H80" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">Rejected by harvest tech</t>
         </is>
       </c>
-      <c r="F80" s="53" t="inlineStr">
+      <c r="I80" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">Passed to our QC</t>
         </is>
       </c>
-      <c r="G80" s="53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QC Pass</t>
-        </is>
-      </c>
-      <c r="H80" s="53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QC Fail</t>
-        </is>
-      </c>
-      <c r="I80" s="53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QC FPY (log basis)</t>
-        </is>
-      </c>
       <c r="J80" s="53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="44" customHeight="1">
+          <t xml:space="preserve">What it took to get the good ones</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="54" customHeight="1">
       <c r="A81" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-08-26</t>
@@ -6870,30 +6870,30 @@
         </is>
       </c>
       <c r="D81" s="55" t="n">
+        <v>8</v>
+      </c>
+      <c r="E81" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" s="56" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="G81" s="55" t="n">
         <v>18</v>
       </c>
-      <c r="E81" s="55" t="n">
+      <c r="H81" s="55" t="n">
         <v>9</v>
       </c>
-      <c r="F81" s="55" t="n">
+      <c r="I81" s="55" t="n">
         <v>9</v>
       </c>
-      <c r="G81" s="55" t="n">
-        <v>8</v>
-      </c>
-      <c r="H81" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="I81" s="56" t="n">
-        <v>0.8889</v>
-      </c>
       <c r="J81" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Harvest-stage rejects included lung/heart lacerations (visit totals: 8 lung, 2 heart; stage split not itemized). 2 upper-vessel-damage blocks passed &amp; labeled for the usability study; rebound credited to Francisco's team.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="44" customHeight="1">
+          <t xml:space="preserve">It took 18 blocks at harvest to get 8 good ones: Jordan rejected 9 while harvesting (lung/heart lacerations; visit totals 8 lung, 2 heart), passed 9 to our QC, and QC rejected 1 more. 2 upper-vessel-damage blocks passed &amp; labeled for the usability study; rebound credited to Francisco's team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="54" customHeight="1">
       <c r="A82" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-09</t>
@@ -6910,26 +6910,26 @@
         </is>
       </c>
       <c r="D82" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" s="56" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G82" s="55" t="n">
         <v>19</v>
       </c>
-      <c r="E82" s="55" t="n">
+      <c r="H82" s="55" t="n">
         <v>17</v>
       </c>
-      <c r="F82" s="55" t="n">
+      <c r="I82" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="G82" s="55" t="n">
-        <v>2</v>
-      </c>
-      <c r="H82" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="I82" s="56" t="n">
-        <v>1.0</v>
-      </c>
       <c r="J82" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Harvest-stage rejects: 8 left-lung lacerations + 9 missing trachea (SH harvesting tracheas for another buyer). One passed unit labeled for a high head-vessel laceration.</t>
+          <t xml:space="preserve">It took 19 blocks at harvest to get 2 good ones: Jordan rejected 17 — 8 left-lung lacerations + 9 missing trachea (SH harvesting tracheas for another buyer). Both blocks passed to our QC were accepted (one labeled for a high head-vessel laceration).</t>
         </is>
       </c>
     </row>
@@ -7259,7 +7259,7 @@
       </c>
       <c r="B113" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">First-pass yield fell 32% (7/29) → 0% (8/5) → 15% (8/12) → 21% (8/19); right-lung perimeter and increasingly heart lacerations dominate (harvesting-side; escalated with Ricardo). The 8/12 pelvic 666541 line reads 13/1/12 with no per-defect breakdown (pelvics deprioritized — Jordan harvests other components first);  UPDATE: the 8/12 pelvic line is UNVERIFIED (no reasons on the source sheet) and is excluded from all defect-profile charts and the Issue Data until confirmed with Kris; it remains in the log, flagged.</t>
+          <t xml:space="preserve">First-pass yield fell 32% (7/29) → 0% (8/5) → 15% (8/12) → 21% (8/19); right-lung perimeter and increasingly heart lacerations dominate (harvesting-side; escalated with Ricardo). The 8/12 pelvic 666541 line (13/1/12) was a PRE-RECEIPT SCREEN: the blocks were inspected prior to receiving them, before the harvesting tech got the tissue (pelvics deprioritized — Jordan harvests other components first). Its 12 rejects are not incoming-QC failures and the line is not FPY-graded; no reasons itemized on the source sheet, so it is excluded from defect-profile views.</t>
         </is>
       </c>
     </row>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="B116" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Former 'Other / unspecified' items now carry their real reasons as named categories: Blood clots (2, 4/15), Handling damage (cleaning) (2, 4/20), Deformed ligaments (1, 5/18), Undocumented / not itemized (7/20 count discrepancy: 1; 8/26 QC-stage fail not stage-itemized: 1). The Nahunta 8/12 pelvic line (13/1/12) is UNVERIFIED — the source sheet recorded totals with no reasons — and is excluded from all defect-profile views (Monthly, month tabs, SH vs ATM Issues) pending confirmation with Kris; it remains in the log and totals, flagged in yellow.</t>
+          <t xml:space="preserve">Former 'Other / unspecified' items now carry their real reasons as named categories: Blood clots (2, 4/15), Handling damage (cleaning) (2, 4/20), Deformed ligaments (1, 5/18), Undocumented / not itemized (7/20 count discrepancy: 1; 8/26 QC-stage fail not stage-itemized: 1). The Nahunta 8/12 pelvic line (13/1/12) was a PRE-RECEIPT SCREEN — inspected prior to receiving them, before the harvesting tech got the tissue; its 12 rejects are not incoming-QC failures, the line is not FPY-graded, and with no reasons itemized it is excluded from all defect-profile views (Monthly, month tabs, SH vs ATM Issues); it remains in the log and totals, flagged in yellow.</t>
         </is>
       </c>
     </row>
@@ -7343,7 +7343,7 @@
     <mergeCell ref="B115:N115"/>
     <mergeCell ref="B116:N116"/>
   </mergeCells>
-  <conditionalFormatting sqref="L6:L70">
+  <conditionalFormatting sqref="L6:L59 L61:L70">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0.3"/>
@@ -10466,7 +10466,7 @@
     <row r="19" ht="44" customHeight="1">
       <c r="A19" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Read: on the same 12 Martins lots, ATM finds ~4× the SH floor-sample fail count (full-batch review vs ~10% sampling). 9972 Laceration/Cut (100) is the downstream face of the SH urethra/bladder &amp; membrane cut damage; Exposed Urethra (16) and Bladder Length (15) map to the same themes; Blood Clots (17) and Spoilage only surface post-freeze.</t>
+          <t xml:space="preserve">Read: on the same 12 Martins lots, ATM finds ~6× the SH floor-sample fail count (full-batch review vs ~10% sampling). 9972 Laceration/Cut (100) is the downstream face of the SH urethra/bladder &amp; membrane cut damage; Exposed Urethra (16) and Bladder Length (15) map to the same themes; Blood Clots (17) and Spoilage only surface post-freeze.</t>
         </is>
       </c>
     </row>
@@ -11189,7 +11189,7 @@
     <row r="66" ht="44" customHeight="1">
       <c r="A66" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">• SH profiles include only verified, categorized fails: the Nahunta 8/12 pelvic line (12 fails, no reasons recorded) is excluded pending confirmation with Kris, and Nahunta harvest-stage rejects (two-inspection visits, from 08/26) are excluded — SH rows reflect our QC inspections. The former 'Other / unspecified' category no longer exists.</t>
+          <t xml:space="preserve">• SH profiles include only incoming-QC fails with verified reasons. Excluded: the Nahunta 8/12 pelvic line (a PRE-RECEIPT SCREEN — 13 blocks inspected prior to receiving them; its 12 rejects never became received product) and Nahunta harvest-stage rejects (two-inspection visits, from 08/26) — SH rows reflect our QC inspections. The former 'Other / unspecified' category no longer exists.</t>
         </is>
       </c>
     </row>
@@ -23853,7 +23853,7 @@
     <row r="25" ht="58" customHeight="1">
       <c r="A25" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Performance-goal part. Steady 94–98% at Martins through August; Parks runs 666541 since 08/10 (95.7% in August). The Nahunta 8/12 line (13/1/12) drags the average and is UNVERIFIED — no scrap reasons on the source sheet; excluded from defect profiles pending confirmation with Kris. Verified rejects: urethra/bladder &amp; membrane damage, short blocks.</t>
+          <t xml:space="preserve">Performance-goal part. Steady 94–98% at Martins through August; Parks runs 666541 since 08/10 (95.7% in August). The Nahunta 8/12 line (13/1/12) was a PRE-RECEIPT SCREEN — inspected prior to receiving them, before the harvesting tech got the tissue; its 12 rejects are not incoming-QC fails and the line is not FPY-graded (excluded from defect profiles). Verified rejects: urethra/bladder &amp; membrane damage, short blocks.</t>
         </is>
       </c>
     </row>
@@ -25643,7 +25643,7 @@
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="60" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 fails recorded (8/12) — UNVERIFIED: no scrap reasons on the source sheet; excluded from defect counts pending confirmation with Kris.</t>
+          <t xml:space="preserve">13 blocks screened on 8/12 PRIOR TO RECEIPT (before the harvesting tech got the tissue); the 12 rejects never became received product and are not incoming-QC fails. Not FPY-graded; no reasons itemized; excluded from defect counts.</t>
         </is>
       </c>
     </row>
@@ -25957,7 +25957,7 @@
     <mergeCell ref="A101:H101"/>
     <mergeCell ref="A102:H102"/>
   </mergeCells>
-  <conditionalFormatting sqref="B6:H11 B27:H27 B42:H42 B57:H57 B71:H71 B82:H82 B90:H90">
+  <conditionalFormatting sqref="B6:H9 B11:H11 B27:H27 B42:H42 B57:H57 B71:H71 B90:H90">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0.3"/>
@@ -26736,7 +26736,7 @@
     <mergeCell ref="A33:J33"/>
     <mergeCell ref="A34:J34"/>
   </mergeCells>
-  <conditionalFormatting sqref="F6:F7">
+  <conditionalFormatting sqref="F6:F6 F7:F7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0.3"/>
@@ -27768,7 +27768,7 @@
     <mergeCell ref="A44:J44"/>
     <mergeCell ref="A45:J45"/>
   </mergeCells>
-  <conditionalFormatting sqref="F6:F8">
+  <conditionalFormatting sqref="F6:F6 F7:F7 F8:F8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0.3"/>
@@ -29029,7 +29029,7 @@
     <mergeCell ref="A49:J49"/>
     <mergeCell ref="A50:J50"/>
   </mergeCells>
-  <conditionalFormatting sqref="F6:F8">
+  <conditionalFormatting sqref="F6:F6 F7:F7 F8:F8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0.3"/>
@@ -30397,7 +30397,7 @@
     <mergeCell ref="A57:J57"/>
     <mergeCell ref="A58:J58"/>
   </mergeCells>
-  <conditionalFormatting sqref="F6:F10">
+  <conditionalFormatting sqref="F6:F6 F7:F7 F8:F8 F9:F9 F10:F10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0.3"/>
@@ -30635,7 +30635,7 @@
       </c>
       <c r="G9" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNVERIFIED — no reasons recorded (see notes)</t>
+          <t xml:space="preserve">Pre-receipt screen — inspected before receipt (see notes)</t>
         </is>
       </c>
     </row>
@@ -30826,7 +30826,7 @@
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pelvic @ Nahunta · 666541 — 12 fails of 13 inspected — UNVERIFIED: no scrap reasons recorded on the source sheet; excluded from defect charts pending confirmation with Kris.</t>
+          <t xml:space="preserve">Pelvic @ Nahunta · 666541 — 12 rejects of 13 screened PRIOR TO RECEIPT (before the harvesting tech got the tissue) — not incoming-QC fails and not FPY-graded; no reasons itemized; excluded from defect charts.</t>
         </is>
       </c>
     </row>
@@ -31315,7 +31315,7 @@
       </c>
       <c r="J41" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNVERIFIED — no scrap reasons recorded on the source sheet (totals only). Pelvics deprioritized on the line (Jordan harvests other components from the blocks). Counts provisional; EXCLUDED from defect-profile charts pending confirmation with Kris.</t>
+          <t xml:space="preserve">PRE-RECEIPT SCREEN — these 13 blocks were inspected prior to receiving them (before the harvesting tech got the tissue); the 12 rejects never became received product, so this line is not graded as incoming first-pass yield. No scrap reasons itemized on the source sheet; excluded from defect-profile charts.</t>
         </is>
       </c>
     </row>
@@ -31799,7 +31799,7 @@
     <row r="57" ht="27.0" customHeight="1">
       <c r="A57" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">➢ 666541 (Pelvic @ Nahunta): the 8/12 line (13 inspected / 12 fail) is UNVERIFIED — no scrap reasons on the source sheet; excluded from defect charts pending confirmation with Kris.</t>
+          <t xml:space="preserve">➢ 666541 (Pelvic @ Nahunta): the 8/12 line (13/1/12) was a PRE-RECEIPT SCREEN — inspected prior to receiving them, before the harvesting tech got the tissue; the 12 rejects never became received product, so it is not graded as incoming FPY (no reasons itemized; excluded from defect charts).</t>
         </is>
       </c>
       <c r="B57" s="47"/>
@@ -31848,7 +31848,7 @@
     <mergeCell ref="A56:J56"/>
     <mergeCell ref="A57:J57"/>
   </mergeCells>
-  <conditionalFormatting sqref="F6:F10">
+  <conditionalFormatting sqref="F6:F6 F7:F7 F8:F8 F10:F10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0.3"/>

</xml_diff>

<commit_message>
Add 'Nahunta Standard' tab: standardized per-visit metrics, future tally spec, data-gap register
Nahunta tallies were collected on three bases (whole-harvest, two-stage
QC-of-passed, pre-receipt screen). New tab restates every visit on Harvest
yield (usable/at-harvest) and QC accept (pass/presented), gives the trend on
the comparable harvest basis (31.6% -> 0 -> 15.4% -> 20.7% -> 44.4% -> 10.5%;
21.2% overall), defines the standard five-number tally for future visits, and
lists 7 open data gaps with owners. Log note 29 points to it; README updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/SH_IQC_Inspections.xlsx
+++ b/QC inspections suppliers/SH_IQC_Inspections.xlsx
@@ -25,6 +25,7 @@
     <sheet name="Jul 2026" sheetId="19" r:id="rId7"/>
     <sheet name="Aug 2026" sheetId="20" r:id="rId8"/>
     <sheet name="Sep 2026" sheetId="24" r:id="rId19"/>
+    <sheet name="Nahunta Standard" sheetId="25" r:id="rId20"/>
     <sheet name="SmartAssessment" sheetId="12" r:id="rId9"/>
     <sheet name="Defect Atlas" sheetId="9" r:id="rId10"/>
     <sheet name="README" sheetId="10" r:id="rId11"/>
@@ -2423,7 +2424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N116"/>
+  <dimension ref="A1:N117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -7290,17 +7291,29 @@
     <row r="116" ht="62.0" customHeight="1">
       <c r="A116" s="58" t="inlineStr">
         <is>
+          <t xml:space="preserve">29. Nahunta standardization</t>
+        </is>
+      </c>
+      <c r="B116" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nahunta's numbers have been collected on three different bases: single-stage whole-harvest tallies (7/29-8/19), two-stage QC-of-harvest-passed tallies (8/26, 9/9), and one pre-receipt screen (8/12 pelvic). The 'Nahunta Standard' tab restates every visit on two standard metrics — Harvest yield (usable blocks / blocks at harvest) and QC accept rate (QC pass / presented to our QC) — defines the standard tally for future visits, and lists the open data gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="62.0" customHeight="1">
+      <c r="A117" s="58" t="inlineStr">
+        <is>
           <t xml:space="preserve">28. Defect categories cleaned; no more 'Other'</t>
         </is>
       </c>
-      <c r="B116" s="59" t="inlineStr">
+      <c r="B117" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">Former 'Other / unspecified' items now carry their real reasons as named categories: Blood clots (2, 4/15), Handling damage (cleaning) (2, 4/20), Deformed ligaments (1, 5/18), Undocumented / not itemized (7/20 count discrepancy: 1; 8/26 QC-stage fail not stage-itemized: 1). The Nahunta 8/12 pelvic line (13/1/12) was a PRE-RECEIPT SCREEN — inspected prior to receiving them, before the harvesting tech got the tissue; its 12 rejects are not incoming-QC failures, the line is not FPY-graded, and with no reasons itemized it is excluded from all defect-profile views (Monthly, month tabs, SH vs ATM Issues); it remains in the log and totals, flagged in yellow.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="42">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A4:N4"/>
@@ -7342,6 +7355,7 @@
     <mergeCell ref="B114:N114"/>
     <mergeCell ref="B115:N115"/>
     <mergeCell ref="B116:N116"/>
+    <mergeCell ref="B117:N117"/>
   </mergeCells>
   <conditionalFormatting sqref="L6:L59 L61:L70">
     <cfRule type="colorScale" priority="1">
@@ -9433,12 +9447,12 @@
       </c>
       <c r="I24" s="53" t="inlineStr">
         <is>
+          <t xml:space="preserve">9983 Incorrect Dimensions</t>
+        </is>
+      </c>
+      <c r="J24" s="53" t="inlineStr">
+        <is>
           <t xml:space="preserve">9978 Damage to Suspensory</t>
-        </is>
-      </c>
-      <c r="J24" s="53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9983 Incorrect Dimensions</t>
         </is>
       </c>
       <c r="K24" s="53" t="inlineStr">
@@ -9545,7 +9559,7 @@
       <c r="E30" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="J30" s="55" t="n">
+      <c r="I30" s="55" t="n">
         <v>1</v>
       </c>
       <c r="K30" s="55" t="n">
@@ -9611,7 +9625,7 @@
       <c r="E33" s="55" t="n">
         <v>11</v>
       </c>
-      <c r="I33" s="55" t="n">
+      <c r="J33" s="55" t="n">
         <v>1</v>
       </c>
       <c r="K33" s="55" t="n">
@@ -23372,6 +23386,787 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K33"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="6" width="12" customWidth="1"/>
+    <col min="7" max="8" width="8" customWidth="1"/>
+    <col min="9" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="46" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nahunta — Standardized View &amp; Data Gaps</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1">
+      <c r="A2" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nahunta's tallies have been collected on THREE different bases — single-stage whole-harvest (7/29–8/19), two-stage QC-of-harvest-passed (8/26, 9/9), and one pre-receipt screen (8/12 pelvic) — so raw FPY figures are not comparable across visits. This tab restates every visit on two standard metrics: HARVEST YIELD = usable blocks / blocks at harvest (comparable across all visits) and QC ACCEPT = QC pass / presented to our QC. It also defines the standard tally for future visits and lists what is still missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">THORACIC 666521 — ALL VISITS, STANDARDIZED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lot</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tally basis</t>
+        </is>
+      </c>
+      <c r="D5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># At harvest</t>
+        </is>
+      </c>
+      <c r="E5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rejected by harvest tech</t>
+        </is>
+      </c>
+      <c r="F5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presented to our QC</t>
+        </is>
+      </c>
+      <c r="G5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC Pass</t>
+        </is>
+      </c>
+      <c r="H5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC Fail</t>
+        </is>
+      </c>
+      <c r="I5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harvest yield</t>
+        </is>
+      </c>
+      <c r="J5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC accept</t>
+        </is>
+      </c>
+      <c r="K5" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reasons (short)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-29</t>
+        </is>
+      </c>
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502512218</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single-stage (whole harvest)</t>
+        </is>
+      </c>
+      <c r="D6" s="55" t="n">
+        <v>19</v>
+      </c>
+      <c r="E6" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— (not recorded)</t>
+        </is>
+      </c>
+      <c r="F6" s="55" t="n">
+        <v>19</v>
+      </c>
+      <c r="G6" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="H6" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="I6" s="56" t="n">
+        <v>0.3158</v>
+      </c>
+      <c r="J6" s="56" t="n">
+        <v>0.3158</v>
+      </c>
+      <c r="K6" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11 right-lung lacerations + 2 heart lacerations</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-05</t>
+        </is>
+      </c>
+      <c r="B7" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502512218</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single-stage (whole harvest)</t>
+        </is>
+      </c>
+      <c r="D7" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— (not recorded)</t>
+        </is>
+      </c>
+      <c r="F7" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="G7" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="I7" s="56" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J7" s="56" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K7" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11 lung + 4 heart lacerations (0% visit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-12</t>
+        </is>
+      </c>
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502523283</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single-stage (whole harvest)</t>
+        </is>
+      </c>
+      <c r="D8" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— (not recorded)</t>
+        </is>
+      </c>
+      <c r="F8" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="G8" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="I8" s="56" t="n">
+        <v>0.1538</v>
+      </c>
+      <c r="J8" s="56" t="n">
+        <v>0.1538</v>
+      </c>
+      <c r="K8" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9 lung + 3 heart recorded — sums 12 vs 11 fails (gap #2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-19</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502523283</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single-stage (whole harvest)</t>
+        </is>
+      </c>
+      <c r="D9" s="55" t="n">
+        <v>29</v>
+      </c>
+      <c r="E9" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— (not recorded)</t>
+        </is>
+      </c>
+      <c r="F9" s="55" t="n">
+        <v>29</v>
+      </c>
+      <c r="G9" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" s="55" t="n">
+        <v>23</v>
+      </c>
+      <c r="I9" s="56" t="n">
+        <v>0.2069</v>
+      </c>
+      <c r="J9" s="56" t="n">
+        <v>0.2069</v>
+      </c>
+      <c r="K9" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11 lung + 12 heart lacerations</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502539375</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two-stage</t>
+        </is>
+      </c>
+      <c r="D10" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="E10" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="G10" s="55" t="n">
+        <v>8</v>
+      </c>
+      <c r="H10" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="56" t="n">
+        <v>0.4444</v>
+      </c>
+      <c r="J10" s="56" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="K10" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visit totals 8 lung + 2 heart; harvest/QC stage split not itemized (gap #3) — the 1 QC fail is undocumented</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502550281</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two-stage</t>
+        </is>
+      </c>
+      <c r="D11" s="55" t="n">
+        <v>19</v>
+      </c>
+      <c r="E11" s="55" t="n">
+        <v>17</v>
+      </c>
+      <c r="F11" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="56" t="n">
+        <v>0.1053</v>
+      </c>
+      <c r="J11" s="56" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="K11" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harvest stage: 8 left-lung lacerations + 9 MISSING TRACHEA (gap #5); QC stage: none</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TOTAL (harvest basis)</t>
+        </is>
+      </c>
+      <c r="D12" s="55" t="n">
+        <v>113</v>
+      </c>
+      <c r="G12" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="I12" s="56" t="n">
+        <v>0.2124</v>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PELVIC 666541 — SIDE LINE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="B15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lot</t>
+        </is>
+      </c>
+      <c r="C15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tally basis</t>
+        </is>
+      </c>
+      <c r="D15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Screened / inspected</t>
+        </is>
+      </c>
+      <c r="E15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+      <c r="F15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="G15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harvest yield</t>
+        </is>
+      </c>
+      <c r="H15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QC accept</t>
+        </is>
+      </c>
+      <c r="I15" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reasons (short)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-29</t>
+        </is>
+      </c>
+      <c r="B16" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502512218</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single-stage (trial)</t>
+        </is>
+      </c>
+      <c r="D16" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="56" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="H16" s="56" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I16" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single trial block, passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-12</t>
+        </is>
+      </c>
+      <c r="B17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502523283</t>
+        </is>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PRE-RECEIPT SCREEN</t>
+        </is>
+      </c>
+      <c r="D17" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="E17" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="F17" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n/a</t>
+        </is>
+      </c>
+      <c r="H17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n/a</t>
+        </is>
+      </c>
+      <c r="I17" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Screened prior to receipt (before the harvesting tech got the tissue); the 12 rejects never became received product. NO REASONS RECORDED (gap #1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TREND READ (harvest-yield basis — the comparable series)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31.6% (7/29) → 0.0% (8/5) → 15.4% (8/12) → 20.7% (8/19) → 44.4% (8/26) → 10.5% (9/9). Overall: 24 usable of 113 at harvest (21.2%). The 8/26 rebound followed Francisco's team engagement; the 9/9 collapse is driven by the missing-trachea arrangement (9 of the 17 harvest rejects), not a quality regression alone. From 8/26 the harvest tech's own screen carries the loss: our QC accepted 88.9–100% of what he passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STANDARD TALLY — USE ON EVERY NAHUNTA VISIT FROM NOW ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1">
+      <c r="A23" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record five things per visit, per part: (1) # blocks at harvest; (2) # rejected by the harvest tech WITH reasons; (3) # presented to our QC; (4) QC pass / fail WITH reasons; (5) lot number. Log convention: the Inspection Log carries the QC-stage numbers (pass/fail of what was presented to us); the harvest stage is recorded on this tab. With those five numbers every visit yields both standard metrics and stays comparable to Martins and Parks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DATA GAPS — WHAT'S MISSING</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="B26" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What's missing</t>
+        </is>
+      </c>
+      <c r="C26" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why it matters</t>
+        </is>
+      </c>
+      <c r="D26" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ask</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="A27" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B27" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/12 pelvic (lot 5502523283): reasons for the 12 pre-receipt rejects, and confirmation none of them were received</t>
+        </is>
+      </c>
+      <c r="G27" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12 units unexplained; the line is excluded from every defect chart until confirmed</t>
+        </is>
+      </c>
+      <c r="K27" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kris</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="B28" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/12 thoracic: 11 fails recorded vs 12 reasons itemized (9 lung + 3 heart)</t>
+        </is>
+      </c>
+      <c r="G28" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one count on the source sheet is wrong</t>
+        </is>
+      </c>
+      <c r="K28" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kris</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1">
+      <c r="A29" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="B29" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/26: split of the 10 laceration reasons between the harvest stage (9 rejects) and our QC stage (1 fail)</t>
+        </is>
+      </c>
+      <c r="G29" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">our only QC fail that visit is currently 'undocumented'</t>
+        </is>
+      </c>
+      <c r="K29" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kris / Jordan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1">
+      <c r="A30" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="B30" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmation that 7/29–8/19 visits were true whole-harvest tallies (no informal pre-screen by the harvest tech)</t>
+        </is>
+      </c>
+      <c r="G30" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">validates the harvest-yield trend series above</t>
+        </is>
+      </c>
+      <c r="K30" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nahunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="B31" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status of the trachea arrangement (tracheas harvested for another buyer)</t>
+        </is>
+      </c>
+      <c r="G31" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">caused 9 of 17 rejects on 9/9; determines whether thoracic supply is viable</t>
+        </is>
+      </c>
+      <c r="K31" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nahunta management</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="B32" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic side-line status — no pelvic inspection since 8/12</t>
+        </is>
+      </c>
+      <c r="G32" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">decides whether pelvic sampling continues at Nahunta</t>
+        </is>
+      </c>
+      <c r="K32" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nahunta</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="B33" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adoption of the standard tally (five numbers above) starting next visit</t>
+        </is>
+      </c>
+      <c r="G33" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">keeps every future visit comparable</t>
+        </is>
+      </c>
+      <c r="K33" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kris + Jordan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G33:J33"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I6:I12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.4"/>
+        <cfvo type="num" val="0.9"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6:J11">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I31"/>

</xml_diff>